<commit_message>
feat: integracion de Mercado Libre y Argenprop - 33 propiedades verificadas multicanal
</commit_message>
<xml_diff>
--- a/data/oportunidades_mendoza.xlsx
+++ b/data/oportunidades_mendoza.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -574,30 +574,30 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>86.7</v>
+        <v>63.3</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>135000</v>
+        <v>94000</v>
       </c>
       <c r="E3" t="n">
-        <v>170</v>
+        <v>109</v>
       </c>
       <c r="F3" t="n">
-        <v>794.1</v>
+        <v>862.4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -627,32 +627,32 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>VENTA CASA 5 AMBIENTES ALTO DORREGO MENDOZA</t>
+          <t>ADOBE INMOBILIARIA VENDE EXCELENTE DÚPLEX EN CALLE TOMBA, GODOY CRUZ</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19363/ficha/casa-en-venta-en-zeballos-500</t>
+          <t>https://www.inmoclick.com.ar/276954-adobe-inmobiliaria-y-desarrollos/inmuebles/318/ficha/departamento-en-venta-en-tomba-35</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 135,000) | 🛡️ Cuenta con seguridad 24 hs / barrio privado | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 94,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>56.2</v>
+        <v>60.9</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -661,17 +661,17 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>63000</v>
+        <v>98000</v>
       </c>
       <c r="E4" t="n">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="F4" t="n">
-        <v>463.2</v>
+        <v>1225</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -696,37 +696,37 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>OPORTUNIDAD EN PLENO CENTRO</t>
+          <t>Coldwell Banker ImpactoPro ofrece en venta departamento en planta baja con patio y cochera en Godoy Cruz,</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/133635-di-luca-propiedades/inmuebles/102/ficha/departamento-en-venta-en-buenos-aires-n0-258-ciudad</t>
+          <t>https://www.inmoclick.com.ar/288316-coldwell-banker-impacto-pro/inmuebles/43/ficha/departamento-en-venta-en-gutierrez-598</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 98,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>55.3</v>
+        <v>56.2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -735,13 +735,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>95000</v>
+        <v>63000</v>
       </c>
       <c r="E5" t="n">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="F5" t="n">
-        <v>871.6</v>
+        <v>463.2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -775,17 +775,17 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>VENTA DEPARTAMENTO – GODOY CRUZ</t>
+          <t>OPORTUNIDAD EN PLENO CENTRO</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1974/ficha/departamento-en-venta-en-avenida-san-martin-100</t>
+          <t>https://www.inmoclick.com.ar/133635-di-luca-propiedades/inmuebles/102/ficha/departamento-en-venta-en-buenos-aires-n0-258-ciudad</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -796,26 +796,26 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>51.6</v>
+        <v>55.3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>120000</v>
+        <v>95000</v>
       </c>
       <c r="E6" t="n">
-        <v>154</v>
+        <v>109</v>
       </c>
       <c r="F6" t="n">
-        <v>779.2</v>
+        <v>871.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -849,17 +849,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>OFRECE EN VENTA</t>
+          <t>VENTA DEPARTAMENTO – GODOY CRUZ</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/18739/ficha/casa-en-venta-en-montevideo-700</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1974/ficha/departamento-en-venta-en-avenida-san-martin-100</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -870,11 +870,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>50.8</v>
+        <v>52.2</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -883,17 +883,17 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>68000</v>
+        <v>90000</v>
       </c>
       <c r="E7" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>906.7</v>
+        <v>900</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No/Duda</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -923,47 +923,47 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>DRUMMOND NEGOCIOS INMOBILIARIOS VENDE</t>
+          <t>ADOBE INMOBILIARIA VENDE  DÚPLEX EN GODOY CRUZ</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/124071-drummond-negocios-inmobiliarios/inmuebles/43/ficha/departamento-en-venta-en-espana-y-gutierrez</t>
+          <t>https://www.inmoclick.com.ar/276954-adobe-inmobiliaria-y-desarrollos/inmuebles/403/ficha/departamento-en-venta-en-perito-moreno-al-500</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 68,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>48.3</v>
+        <v>51.6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>130000</v>
+        <v>120000</v>
       </c>
       <c r="E8" t="n">
-        <v>75</v>
+        <v>154</v>
       </c>
       <c r="F8" t="n">
-        <v>1733.3</v>
+        <v>779.2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -997,17 +997,17 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>"CARINA DROZD gestiones inmobiliarias" VENDE: DEPARTAMENTOS Ubicadísimos: Calle ALMIRANTE BROWN, B° BOMBAL SUR. Complejo de 7 deptos con cocheras subterráneas. ASCENSOR. Piso 1 y Piso 2. FRONTALES!. Constan de: COCINA LIVING COMEDOR con Equipo A.A. y Calefactor; cocina con extractor, alacenas, bajomesada, Barra Desayunador- 2 DORMITORIOS (1 con A.A.) con Placares y Calefactores- 2 BAÑOS (uno en SUITE)- Recién Pintados! BALCON- PATIO LAVANDERÍA con bacha y mueble- COCHERA AUTOMATIZADA, en Subsuelo. VALORES: U$S 115.000 sin cochera en Piso 1- U$S 130.000 con Cochera en Piso 2. ESCRITURACION Inmediata. ALQUILADOS con Excelentes Rentas, pero se desocupan si lo desea el comprador-</t>
+          <t>OFRECE EN VENTA</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/1406-carina-drozd-gestiones-inmobiliarias/inmuebles/3601/ficha/departamento-en-venta-en-almirante-brown-1524</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/18739/ficha/casa-en-venta-en-montevideo-700</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1018,7 +1018,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>48.1</v>
+        <v>50.8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1031,17 +1031,17 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>63000</v>
+        <v>68000</v>
       </c>
       <c r="E9" t="n">
-        <v>112</v>
+        <v>75</v>
       </c>
       <c r="F9" t="n">
-        <v>562.5</v>
+        <v>906.7</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1071,22 +1071,22 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Oportunidad de inversión!</t>
+          <t>DRUMMOND NEGOCIOS INMOBILIARIOS VENDE</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/259304-bcg-desarrollos-inmobiliarios/inmuebles/28/ficha/departamento-en-venta-en-pte-derqui-243</t>
+          <t>https://www.inmoclick.com.ar/124071-drummond-negocios-inmobiliarios/inmuebles/43/ficha/departamento-en-venta-en-espana-y-gutierrez</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 68,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1105,13 +1105,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>75000</v>
+        <v>63000</v>
       </c>
       <c r="E10" t="n">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="F10" t="n">
-        <v>1000</v>
+        <v>562.5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1145,17 +1145,17 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
+          <t>Oportunidad de inversión!</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
+          <t>https://www.inmoclick.com.ar/259304-bcg-desarrollos-inmobiliarios/inmuebles/28/ficha/departamento-en-venta-en-pte-derqui-243</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1166,7 +1166,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>47.7</v>
+        <v>48.1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>86000</v>
+        <v>75000</v>
       </c>
       <c r="E11" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F11" t="n">
-        <v>1228.6</v>
+        <v>1000</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1219,17 +1219,17 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
+          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
+          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1240,7 +1240,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>45.3</v>
+        <v>47.7</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1253,13 +1253,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>79000</v>
+        <v>86000</v>
       </c>
       <c r="E12" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="F12" t="n">
-        <v>718.2</v>
+        <v>1228.6</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1293,17 +1293,17 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Bombal Sur. Piso completo - Beltran 1.910 esquina 25 de Mayo. Excelente ubicacion geografica. Cerca Estacion Metrotanvia. Limite con Barrio Bombal de Ciudad. 2° Piso. Muy luminoso . Living comedor amplio. Cocina comedor mediana. 3 dormitorios con placares. 2 baños. Ascensor .Apto Credito . Desocupado. Javier / Armando</t>
+          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/16797-provivienda-inmobiliaria/inmuebles/811/ficha/departamento-en-venta-en-beltran-1-910</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 79,000) | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1314,7 +1314,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>45.2</v>
+        <v>46.6</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1327,13 +1327,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>140000</v>
+        <v>90000</v>
       </c>
       <c r="E13" t="n">
-        <v>575</v>
+        <v>96</v>
       </c>
       <c r="F13" t="n">
-        <v>243.5</v>
+        <v>937.5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1367,17 +1367,17 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>OPENHOUSE vende desarrollo en obra gruesa sobre calle Pascual Segura de Godoy Cruz</t>
+          <t>Departamento en Venta en Godoy Cruz</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2063/ficha/departamento-en-venta-en-pascual-segura-godoy-cruz</t>
+          <t>https://www.inmoclick.com.ar/259304-bcg-desarrollos-inmobiliarios/inmuebles/22/ficha/departamento-en-venta-en-san-martin-1338</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1462,11 +1462,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>39.9</v>
+        <v>41.4</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1475,13 +1475,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>70000</v>
+        <v>85000</v>
       </c>
       <c r="E15" t="n">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="F15" t="n">
-        <v>1000</v>
+        <v>904.3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Venta de Departamento – Cuarta Sección Oeste</t>
+          <t>Venta departamento en Godoy Cruz planta baja apto crédito 3 dormitorios reciclado</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/3076-ente-inmobiliaria/inmuebles/3329/ficha/departamento-en-venta-en-fray-inalican-363</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19508/ficha/departamento-en-venta-en-salta-400</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 70,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 85,000)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1536,7 +1536,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>39.8</v>
+        <v>39.9</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1549,13 +1549,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>140000</v>
+        <v>70000</v>
       </c>
       <c r="E16" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F16" t="n">
-        <v>1866.7</v>
+        <v>1000</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1589,17 +1589,17 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Departamento en Venta – Mendoza Capital</t>
+          <t>Venta de Departamento – Cuarta Sección Oeste</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/276253-sere-inmobiliaria/inmuebles/136/ficha/departamento-en-venta-en-peatonal-y-9-de-julio</t>
+          <t>https://www.inmoclick.com.ar/3076-ente-inmobiliaria/inmuebles/3329/ficha/departamento-en-venta-en-fray-inalican-363</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 70,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>130000</v>
+        <v>140000</v>
       </c>
       <c r="E17" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" t="n">
-        <v>1756.8</v>
+        <v>1866.7</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1663,17 +1663,17 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO  ubicado sobre calle Huarpes 2046 - Sexta Sección - Mendoza.</t>
+          <t>Departamento en Venta – Mendoza Capital</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/844/ficha/departamento-en-venta-en-sexta-seccion-ciudad-mendoza</t>
+          <t>https://www.inmoclick.com.ar/276253-sere-inmobiliaria/inmuebles/136/ficha/departamento-en-venta-en-peatonal-y-9-de-julio</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1684,7 +1684,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>36.6</v>
+        <v>39.8</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1697,13 +1697,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>98000</v>
+        <v>130000</v>
       </c>
       <c r="E18" t="n">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="F18" t="n">
-        <v>890.9</v>
+        <v>1756.8</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1737,17 +1737,17 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>SCAFFIDI PROPIEDADES VENDE</t>
+          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO  ubicado sobre calle Huarpes 2046 - Sexta Sección - Mendoza.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12373-scaffidi-propiedades/inmuebles/269/ficha/departamento-en-venta-en-mitre-565</t>
+          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/844/ficha/departamento-en-venta-en-sexta-seccion-ciudad-mendoza</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 98,000)</t>
+          <t>Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1758,7 +1758,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>36.5</v>
+        <v>37.3</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1774,10 +1774,10 @@
         <v>90000</v>
       </c>
       <c r="E19" t="n">
-        <v>103</v>
+        <v>137</v>
       </c>
       <c r="F19" t="n">
-        <v>873.8</v>
+        <v>656.9</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>SOPPELSA INMOBILIARIA VENDE amplio Departamento en ciudad. Calle Gutiérrez y Mitre. Semipiso de doble ingreso, Ubicado en 5to Piso. Posee Living comedor con Balcón. Cocina comedor amplia. Dependencia de servicio con Baño. 3 Dormitorios. Baño principal y Toilette.</t>
+          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12197-soppelsa-inmobiliaria/inmuebles/397/ficha/departamento-en-venta-en-gutierrez-466-5to-piso</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1832,11 +1832,11 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>35</v>
+        <v>37.2</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1848,10 +1848,10 @@
         <v>90000</v>
       </c>
       <c r="E20" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="F20" t="n">
-        <v>1097.6</v>
+        <v>1363.6</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1885,17 +1885,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Vendo Departamento en Ciudad de Mendoza. 82 mtrs terreno total. La propiedad cuenta con cocina comedor, living, 3 habitaciones, placares, 2 baños, aire acondicionado, calefactores. Los principales ventanales dan a la cordillera. En pleno centro de Mendoza. Se evalúan ofertas. Zelta Inmobiliaria</t>
+          <t>En el corazón del Barrio Bombal, se encuentra este hermoso departamento en planta alta por escalera. Con una superficie total de 80 metros cuadrados y 66 metros cubiertos, cuenta con dos dormitorios, el principal con baño en suite zonificado, y un balcón que proporciona excelente ventilación e iluminación natural. La propiedad no posee gas, siendo todo eléctrico, lo que garantiza un ambiente seguro y eficiente.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/302127-zelta-inmobiliaria/inmuebles/95/ficha/departamento-en-venta-en-catamarca-35</t>
+          <t>https://www.inmoclick.com.ar/4201-vanina-rubio/inmuebles/258/ficha/departamento-en-venta-en-roque-saenz-pena-2051</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000)</t>
+          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -1906,7 +1906,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>34.9</v>
+        <v>36.6</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1919,13 +1919,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>77500</v>
+        <v>98000</v>
       </c>
       <c r="E21" t="n">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="F21" t="n">
-        <v>1174.2</v>
+        <v>890.9</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1959,22 +1959,980 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Follow ofrece en venta un amplio departamento de 3 dormitorios, totalmente refaccionado, ubicado sobre calle Amigorena, en pleno centro de la Ciudad de Mendoza.</t>
+          <t>SCAFFIDI PROPIEDADES VENDE</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/274909-remax-follow/inmuebles/2357/ficha/departamento-en-venta-en-amigorena-0</t>
+          <t>https://www.inmoclick.com.ar/12373-scaffidi-propiedades/inmuebles/269/ficha/departamento-en-venta-en-mitre-565</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 77,500) | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 98,000)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
           <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>58000</v>
+      </c>
+      <c r="E22" t="n">
+        <v>100</v>
+      </c>
+      <c r="F22" t="n">
+        <v>580</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Duplex En Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 58,000)</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E23" t="n">
+        <v>103</v>
+      </c>
+      <c r="F23" t="n">
+        <v>873.8</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>SOPPELSA INMOBILIARIA VENDE amplio Departamento en ciudad. Calle Gutiérrez y Mitre. Semipiso de doble ingreso, Ubicado en 5to Piso. Posee Living comedor con Balcón. Cocina comedor amplia. Dependencia de servicio con Baño. 3 Dormitorios. Baño principal y Toilette.</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/12197-soppelsa-inmobiliaria/inmuebles/397/ficha/departamento-en-venta-en-gutierrez-466-5to-piso</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 90,000)</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E24" t="n">
+        <v>90</v>
+      </c>
+      <c r="F24" t="n">
+        <v>888.9</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 80,000)</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Guaymallen</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>55000</v>
+      </c>
+      <c r="E25" t="n">
+        <v>88</v>
+      </c>
+      <c r="F25" t="n">
+        <v>625</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 55,000)</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>99000</v>
+      </c>
+      <c r="E26" t="n">
+        <v>93</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1064.5</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Venta Amplio Departamento Godoy Cruz  Apto Credito</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3912396714-venta-amplio-departamento-godoy-cruz-apto-credito-_JM</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 99,000)</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Guaymallen</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>110000</v>
+      </c>
+      <c r="E27" t="n">
+        <v>100</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Departamento En Coronel Dorrego</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 110,000)</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>34</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Guaymallen</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>120000</v>
+      </c>
+      <c r="E28" t="n">
+        <v>90</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1333.3</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Departamento Premium De 2 Dormitorios 2 Baños Y Amenitis. En Dorrego Guaymallen</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2052069609-departamento-premium-de-2-dormitorios-2-banos-y-amenitis-en-dorrego-guaymallen-_JM</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 120,000)</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>124900</v>
+      </c>
+      <c r="E29" t="n">
+        <v>87</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1435.6</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Venta Hermoso Departamento Duplex - Barrio Bombal</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1945076259-venta-hermoso-departamento-duplex-barrio-bombal-_JM</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 124,900)</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>128000</v>
+      </c>
+      <c r="E30" t="n">
+        <v>87</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1471.3</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Venta Duplex En Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 128,000)</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>63300</v>
+      </c>
+      <c r="E31" t="n">
+        <v>73</v>
+      </c>
+      <c r="F31" t="n">
+        <v>867.1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Departamento En Gobernador Benegas</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 63,300)</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E32" t="n">
+        <v>74</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2027</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Moderada</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Venta Departamento Godoy Cruz Con Cochera</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1805521295-venta-departamento-godoy-cruz-con-cochera-_JM</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>86000</v>
+      </c>
+      <c r="E33" t="n">
+        <v>71</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1211.3</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Venta Departamento Godoy Cruz. Complejo Privado. Dto 11</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1746780419-venta-departamento-godoy-cruz-complejo-privado-dto-11-_JM</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 86,000)</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E34" t="n">
+        <v>79</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1898.7</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Moderada</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: penalizacion Godoy Cruz fuera de Bombal y priorizacion de novedades en email
</commit_message>
<xml_diff>
--- a/data/oportunidades_mendoza.xlsx
+++ b/data/oportunidades_mendoza.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>91.5</v>
+        <v>82.2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -513,13 +513,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>89999</v>
+        <v>100000</v>
       </c>
       <c r="E2" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>818.2</v>
+        <v>1000</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -553,17 +553,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Departamento en Microcentro en Venta – 3 Dormitorios / 2 Baños / Cochera/ Amoblado</t>
+          <t>DEPARTAMENTO 3 AMBIENTES EN VENTA EN 25 DE MAYO, MENDOZA CAPITAL</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/20134/ficha/departamento-en-venta-en-corrientes-100</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19405/ficha/departamento-en-venta-en-25-de-mayo-900</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 89,999) | 🛡️ Cuenta con seguridad 24 hs / barrio privado | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 100,000) | 🛡️ Cuenta con seguridad 24 hs / barrio privado | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -574,7 +574,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>56.2</v>
+        <v>51.6</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -583,17 +583,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>63000</v>
+        <v>120000</v>
       </c>
       <c r="E3" t="n">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="F3" t="n">
-        <v>463.2</v>
+        <v>779.2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -627,17 +627,17 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>OPORTUNIDAD EN PLENO CENTRO</t>
+          <t>OFRECE EN VENTA</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/133635-di-luca-propiedades/inmuebles/102/ficha/departamento-en-venta-en-buenos-aires-n0-258-ciudad</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/18739/ficha/casa-en-venta-en-montevideo-700</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -648,7 +648,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>55.3</v>
+        <v>48.3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -661,13 +661,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>95000</v>
+        <v>130000</v>
       </c>
       <c r="E4" t="n">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
-        <v>871.6</v>
+        <v>1733.3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -701,17 +701,17 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>VENTA DEPARTAMENTO – GODOY CRUZ</t>
+          <t>"CARINA DROZD gestiones inmobiliarias" VENDE: DEPARTAMENTOS Ubicadísimos: Calle ALMIRANTE BROWN, B° BOMBAL SUR. Complejo de 7 deptos con cocheras subterráneas. ASCENSOR. Piso 1 y Piso 2. FRONTALES!. Constan de: COCINA LIVING COMEDOR con Equipo A.A. y Calefactor; cocina con extractor, alacenas, bajomesada, Barra Desayunador- 2 DORMITORIOS (1 con A.A.) con Placares y Calefactores- 2 BAÑOS (uno en SUITE)- Recién Pintados! BALCON- PATIO LAVANDERÍA con bacha y mueble- COCHERA AUTOMATIZADA, en Subsuelo. VALORES: U$S 115.000 sin cochera en Piso 1- U$S 130.000 con Cochera en Piso 2. ESCRITURACION Inmediata. ALQUILADOS con Excelentes Rentas, pero se desocupan si lo desea el comprador-</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1974/ficha/departamento-en-venta-en-avenida-san-martin-100</t>
+          <t>https://www.inmoclick.com.ar/1406-carina-drozd-gestiones-inmobiliarias/inmuebles/3601/ficha/departamento-en-venta-en-almirante-brown-1524</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -722,7 +722,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>51.6</v>
+        <v>45.7</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -731,17 +731,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>120000</v>
-      </c>
-      <c r="E5" t="n">
-        <v>154</v>
-      </c>
-      <c r="F5" t="n">
-        <v>779.2</v>
+        <v>140000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -775,17 +779,17 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>OFRECE EN VENTA</t>
+          <t>OPENHOUSE VENDE | Exclusivos departamentos en pozo – Quinta Sección</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/18739/ficha/casa-en-venta-en-montevideo-700</t>
+          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2240/ficha/departamento-en-venta-en-5ta-seccion</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -796,11 +800,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>50.8</v>
+        <v>45.3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -809,22 +813,22 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>68000</v>
+        <v>79000</v>
       </c>
       <c r="E6" t="n">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="F6" t="n">
-        <v>906.7</v>
+        <v>718.2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No/Duda</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -849,32 +853,32 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>DRUMMOND NEGOCIOS INMOBILIARIOS VENDE</t>
+          <t>Bombal Sur. Piso completo - Beltran 1.910 esquina 25 de Mayo. Excelente ubicacion geografica. Cerca Estacion Metrotanvia. Limite con Barrio Bombal de Ciudad. 2° Piso. Muy luminoso . Living comedor amplio. Cocina comedor mediana. 3 dormitorios con placares. 2 baños. Ascensor .Apto Credito . Desocupado. Javier / Armando</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/124071-drummond-negocios-inmobiliarios/inmuebles/43/ficha/departamento-en-venta-en-espana-y-gutierrez</t>
+          <t>https://www.inmoclick.com.ar/16797-provivienda-inmobiliaria/inmuebles/811/ficha/departamento-en-venta-en-beltran-1-910</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 68,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 79,000) | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>48.3</v>
+        <v>44.6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -883,13 +887,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>130000</v>
+        <v>90000</v>
       </c>
       <c r="E7" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F7" t="n">
-        <v>1733.3</v>
+        <v>1384.6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -923,17 +927,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>"CARINA DROZD gestiones inmobiliarias" VENDE: DEPARTAMENTOS Ubicadísimos: Calle ALMIRANTE BROWN, B° BOMBAL SUR. Complejo de 7 deptos con cocheras subterráneas. ASCENSOR. Piso 1 y Piso 2. FRONTALES!. Constan de: COCINA LIVING COMEDOR con Equipo A.A. y Calefactor; cocina con extractor, alacenas, bajomesada, Barra Desayunador- 2 DORMITORIOS (1 con A.A.) con Placares y Calefactores- 2 BAÑOS (uno en SUITE)- Recién Pintados! BALCON- PATIO LAVANDERÍA con bacha y mueble- COCHERA AUTOMATIZADA, en Subsuelo. VALORES: U$S 115.000 sin cochera en Piso 1- U$S 130.000 con Cochera en Piso 2. ESCRITURACION Inmediata. ALQUILADOS con Excelentes Rentas, pero se desocupan si lo desea el comprador-</t>
+          <t>Departamento ubicado en 5° piso de Avenida Pedro Molina, Segunda sección de Capital.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/1406-carina-drozd-gestiones-inmobiliarias/inmuebles/3601/ficha/departamento-en-venta-en-almirante-brown-1524</t>
+          <t>https://www.inmoclick.com.ar/105122-helga-kruls-propiedades/inmuebles/121/ficha/departamento-en-venta-en-pedro-molina-461</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -944,11 +948,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>48.1</v>
+        <v>40.3</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -957,13 +961,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>63000</v>
+        <v>95000</v>
       </c>
       <c r="E8" t="n">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F8" t="n">
-        <v>562.5</v>
+        <v>871.6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -997,32 +1001,32 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Oportunidad de inversión!</t>
+          <t>VENTA DEPARTAMENTO – GODOY CRUZ</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/259304-bcg-desarrollos-inmobiliarios/inmuebles/28/ficha/departamento-en-venta-en-pte-derqui-243</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1974/ficha/departamento-en-venta-en-avenida-san-martin-100</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>48.1</v>
+        <v>38.4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1031,22 +1035,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>75000</v>
+        <v>55000</v>
       </c>
       <c r="E9" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F9" t="n">
-        <v>1000</v>
+        <v>763.9</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1071,32 +1075,32 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
+          <t>DEPARTAMENTO DE 4 AMBIENTES - CENTRICO</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
+          <t>https://www.inmoclick.com.ar/68264-gaustralinmobiliariaatgmail-com/inmuebles/4/ficha/departamento-en-venta-en-rondeau</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 55,000) | 🔥 Red de gas natural confirmada</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>47.7</v>
+        <v>37.3</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1105,13 +1109,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>86000</v>
+        <v>90000</v>
       </c>
       <c r="E10" t="n">
-        <v>70</v>
+        <v>137</v>
       </c>
       <c r="F10" t="n">
-        <v>1228.6</v>
+        <v>656.9</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1120,7 +1124,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1145,17 +1149,17 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
+          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 90,000)</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1166,11 +1170,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>45.3</v>
+        <v>35.7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1179,13 +1183,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>79000</v>
+        <v>55000</v>
       </c>
       <c r="E11" t="n">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="F11" t="n">
-        <v>718.2</v>
+        <v>625</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1219,17 +1223,17 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Bombal Sur. Piso completo - Beltran 1.910 esquina 25 de Mayo. Excelente ubicacion geografica. Cerca Estacion Metrotanvia. Limite con Barrio Bombal de Ciudad. 2° Piso. Muy luminoso . Living comedor amplio. Cocina comedor mediana. 3 dormitorios con placares. 2 baños. Ascensor .Apto Credito . Desocupado. Javier / Armando</t>
+          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/16797-provivienda-inmobiliaria/inmuebles/811/ficha/departamento-en-venta-en-beltran-1-910</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 79,000) | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 55,000)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1240,11 +1244,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>45.2</v>
+        <v>35.3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1253,13 +1257,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>140000</v>
+        <v>110000</v>
       </c>
       <c r="E12" t="n">
-        <v>575</v>
+        <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>243.5</v>
+        <v>1100</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1268,7 +1272,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1293,17 +1297,17 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>OPENHOUSE vende desarrollo en obra gruesa sobre calle Pascual Segura de Godoy Cruz</t>
+          <t>Departamento En Coronel Dorrego</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2063/ficha/departamento-en-venta-en-pascual-segura-godoy-cruz</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 110,000)</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1314,7 +1318,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>43.4</v>
+        <v>35.1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1327,13 +1331,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>95000</v>
+        <v>70000</v>
       </c>
       <c r="E13" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F13" t="n">
-        <v>1233.8</v>
+        <v>875</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1342,7 +1346,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1367,17 +1371,17 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Departamento ubicado en una zona estratégica, a poca distancia de Plaza Independencia: una propuesta ideal para quienes buscan comodidad y funcionalidad en el centro. Se trata de un 1° piso frontal que ofrece ambientes bien distribuidos y posibilidades para adaptarlo según tus necesidades.</t>
+          <t>📍 En pleno corazón de la ciudad de Mendoza, este amplio departamento amoblado ofrece comodidad y practicidad en una ubicación difícil de igualar. Espacios bien distribuidos que invitan a sentirse en casa desde el primer momento: cocina funcional, estar-comedor acogedor y dos dormitorios que garantizan privacidad. El mobiliario incluido —camas, mesas de luz, comedor y sala con TV— permite mudarse sin preocupaciones, y la opción de alquiler sin muebles brinda flexibilidad según tus necesidades.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/11968-inmobiliaria-miguel-angel-juan-pablo-simon/inmuebles/51/ficha/departamento-en-venta-en-gutierrez-434</t>
+          <t>https://www.inmoclick.com.ar/311442-plus-valor/inmuebles/2/ficha/departamento-en-venta-en-9-de-julio-1570</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 70,000)</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1388,7 +1392,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>39.9</v>
+        <v>34.6</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1401,13 +1405,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>70000</v>
+        <v>53000</v>
       </c>
       <c r="E14" t="n">
         <v>70</v>
       </c>
       <c r="F14" t="n">
-        <v>1000</v>
+        <v>757.1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1416,7 +1420,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1441,17 +1445,17 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Venta de Departamento – Cuarta Sección Oeste</t>
+          <t>Planta baja confortable y funcional en excelente zona de Dorrego, entre las calles Laprida y Cobos, adyacencias calle Lamadrid, ideal para quienes buscan comodidad, privacidad y ubicación estratégica. Un hogar pensado para el día a día: living comedor para recibir visitas, cocina comedor práctica para las comidas diarias y una lavandería independiente que facilita las tareas del hogar. Tres dormitorios bien distribuidos: dos con placares y un tercero en suite con su propio placard, que ofrece mayor privacidad y confort.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/3076-ente-inmobiliaria/inmuebles/3329/ficha/departamento-en-venta-en-fray-inalican-363</t>
+          <t>https://www.inmoclick.com.ar/308706-cm/inmuebles/6/ficha/departamento-en-venta-en-laprida-y-cobos</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 70,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 53,000)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1462,11 +1466,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>39.8</v>
+        <v>34</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1475,13 +1479,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>140000</v>
+        <v>120000</v>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="F15" t="n">
-        <v>1866.7</v>
+        <v>1333.3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1490,7 +1494,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1515,17 +1519,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Departamento en Venta – Mendoza Capital</t>
+          <t>Departamento Premium De 2 Dormitorios 2 Baños Y Amenitis. En Dorrego Guaymallen</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/276253-sere-inmobiliaria/inmuebles/136/ficha/departamento-en-venta-en-peatonal-y-9-de-julio</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2052069609-departamento-premium-de-2-dormitorios-2-banos-y-amenitis-en-dorrego-guaymallen-_JM</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 120,000)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1536,11 +1540,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>39.8</v>
+        <v>33.5</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1549,13 +1553,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>130000</v>
+        <v>124900</v>
       </c>
       <c r="E16" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="F16" t="n">
-        <v>1756.8</v>
+        <v>1435.6</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1564,7 +1568,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1589,17 +1593,17 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO  ubicado sobre calle Huarpes 2046 - Sexta Sección - Mendoza.</t>
+          <t>Venta Hermoso Departamento Duplex - Barrio Bombal</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/844/ficha/departamento-en-venta-en-sexta-seccion-ciudad-mendoza</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1945076259-venta-hermoso-departamento-duplex-barrio-bombal-_JM</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 124,900)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1610,11 +1614,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>37.3</v>
+        <v>33.1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1623,13 +1627,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>90000</v>
+        <v>75000</v>
       </c>
       <c r="E17" t="n">
-        <v>137</v>
+        <v>75</v>
       </c>
       <c r="F17" t="n">
-        <v>656.9</v>
+        <v>1000</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1638,7 +1642,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1663,32 +1667,32 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
+          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
+          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000)</t>
+          <t>Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>36.6</v>
+        <v>32.7</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1697,13 +1701,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>98000</v>
+        <v>86000</v>
       </c>
       <c r="E18" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="F18" t="n">
-        <v>890.9</v>
+        <v>1228.6</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1712,7 +1716,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1737,28 +1741,28 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>SCAFFIDI PROPIEDADES VENDE</t>
+          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12373-scaffidi-propiedades/inmuebles/269/ficha/departamento-en-venta-en-mitre-565</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 98,000)</t>
+          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>36.6</v>
+        <v>30.2</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1771,13 +1775,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>58000</v>
+        <v>140000</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>575</v>
       </c>
       <c r="F19" t="n">
-        <v>580</v>
+        <v>243.5</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1786,7 +1790,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1811,32 +1815,32 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Duplex En Godoy Cruz</t>
+          <t>OPENHOUSE vende desarrollo en obra gruesa sobre calle Pascual Segura de Godoy Cruz</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
+          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2063/ficha/departamento-en-venta-en-pascual-segura-godoy-cruz</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 58,000)</t>
+          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>36.5</v>
+        <v>21.6</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1845,13 +1849,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>90000</v>
+        <v>58000</v>
       </c>
       <c r="E20" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F20" t="n">
-        <v>873.8</v>
+        <v>580</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1885,28 +1889,28 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>SOPPELSA INMOBILIARIA VENDE amplio Departamento en ciudad. Calle Gutiérrez y Mitre. Semipiso de doble ingreso, Ubicado en 5to Piso. Posee Living comedor con Balcón. Cocina comedor amplia. Dependencia de servicio con Baño. 3 Dormitorios. Baño principal y Toilette.</t>
+          <t>Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12197-soppelsa-inmobiliaria/inmuebles/397/ficha/departamento-en-venta-en-gutierrez-466-5to-piso</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000)</t>
+          <t>Dentro del presupuesto (USD 58,000)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>35.9</v>
+        <v>20.9</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1974,17 +1978,17 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>35.7</v>
+        <v>20.3</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1993,13 +1997,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>55000</v>
+        <v>99000</v>
       </c>
       <c r="E22" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F22" t="n">
-        <v>625</v>
+        <v>1064.5</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2033,28 +2037,28 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
+          <t>Venta Amplio Departamento Godoy Cruz  Apto Credito</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3912396714-venta-amplio-departamento-godoy-cruz-apto-credito-_JM</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 55,000)</t>
+          <t>Dentro del presupuesto (USD 99,000)</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>35.3</v>
+        <v>20</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2067,13 +2071,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>99000</v>
+        <v>150000</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="F23" t="n">
-        <v>1064.5</v>
+        <v>2027</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2082,7 +2086,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2102,37 +2106,37 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Venta Amplio Departamento Godoy Cruz  Apto Credito</t>
+          <t>Venta Departamento Godoy Cruz Con Cochera</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3912396714-venta-amplio-departamento-godoy-cruz-apto-credito-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1805521295-venta-departamento-godoy-cruz-con-cochera-_JM</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 99,000)</t>
+          <t>🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>35.3</v>
+        <v>20</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2141,13 +2145,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>110000</v>
+        <v>86000</v>
       </c>
       <c r="E24" t="n">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="F24" t="n">
-        <v>1100</v>
+        <v>1211.3</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2181,32 +2185,32 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Departamento En Coronel Dorrego</t>
+          <t>Venta Departamento Godoy Cruz. Complejo Privado. Dto 11</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1746780419-venta-departamento-godoy-cruz-complejo-privado-dto-11-_JM</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 110,000)</t>
+          <t>Dentro del presupuesto (USD 86,000)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>34.9</v>
+        <v>20</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2215,13 +2219,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>77500</v>
+        <v>63300</v>
       </c>
       <c r="E25" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F25" t="n">
-        <v>1174.2</v>
+        <v>867.1</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2255,32 +2259,32 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Follow ofrece en venta un amplio departamento de 3 dormitorios, totalmente refaccionado, ubicado sobre calle Amigorena, en pleno centro de la Ciudad de Mendoza.</t>
+          <t>Departamento En Gobernador Benegas</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/274909-remax-follow/inmuebles/2357/ficha/departamento-en-venta-en-amigorena-0</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 77,500) | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 63,300)</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2289,13 +2293,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>120000</v>
+        <v>150000</v>
       </c>
       <c r="E26" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F26" t="n">
-        <v>1333.3</v>
+        <v>1898.7</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2324,33 +2328,29 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Departamento Premium De 2 Dormitorios 2 Baños Y Amenitis. En Dorrego Guaymallen</t>
+          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2052069609-departamento-premium-de-2-dormitorios-2-banos-y-amenitis-en-dorrego-guaymallen-_JM</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 120,000)</t>
-        </is>
-      </c>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>33.5</v>
+        <v>20</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2363,13 +2363,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>124900</v>
+        <v>128000</v>
       </c>
       <c r="E27" t="n">
         <v>87</v>
       </c>
       <c r="F27" t="n">
-        <v>1435.6</v>
+        <v>1471.3</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2403,388 +2403,22 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Venta Hermoso Departamento Duplex - Barrio Bombal</t>
+          <t>Venta Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1945076259-venta-hermoso-departamento-duplex-barrio-bombal-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 124,900)</t>
+          <t>Dentro del presupuesto (USD 128,000)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>128000</v>
-      </c>
-      <c r="E28" t="n">
-        <v>87</v>
-      </c>
-      <c r="F28" t="n">
-        <v>1471.3</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>Venta Duplex En Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 128,000)</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>63300</v>
-      </c>
-      <c r="E29" t="n">
-        <v>73</v>
-      </c>
-      <c r="F29" t="n">
-        <v>867.1</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>Departamento En Gobernador Benegas</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 63,300)</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>150000</v>
-      </c>
-      <c r="E30" t="n">
-        <v>74</v>
-      </c>
-      <c r="F30" t="n">
-        <v>2027</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>Moderada</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>Venta Departamento Godoy Cruz Con Cochera</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1805521295-venta-departamento-godoy-cruz-con-cochera-_JM</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>🚗 Cuenta con cochera</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>86000</v>
-      </c>
-      <c r="E31" t="n">
-        <v>71</v>
-      </c>
-      <c r="F31" t="n">
-        <v>1211.3</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>Venta Departamento Godoy Cruz. Complejo Privado. Dto 11</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1746780419-venta-departamento-godoy-cruz-complejo-privado-dto-11-_JM</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 86,000)</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>150000</v>
-      </c>
-      <c r="E32" t="n">
-        <v>79</v>
-      </c>
-      <c r="F32" t="n">
-        <v>1898.7</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>Moderada</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: minimo 2 dormitorios y 3 ambientes excluyente, bonus por dormitorios extra y resumen visual de configuracion en el email
</commit_message>
<xml_diff>
--- a/data/oportunidades_mendoza.xlsx
+++ b/data/oportunidades_mendoza.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>82.2</v>
+        <v>96.7</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -509,17 +509,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>100000</v>
+        <v>135000</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>170</v>
       </c>
       <c r="F2" t="n">
-        <v>1000</v>
+        <v>794.1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -553,17 +553,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO 3 AMBIENTES EN VENTA EN 25 DE MAYO, MENDOZA CAPITAL</t>
+          <t>VENTA CASA 5 AMBIENTES ALTO DORREGO MENDOZA</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19405/ficha/departamento-en-venta-en-25-de-mayo-900</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19363/ficha/casa-en-venta-en-zeballos-500</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 100,000) | 🛡️ Cuenta con seguridad 24 hs / barrio privado | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 135,000) | 🛡️ Cuenta con seguridad 24 hs / barrio privado | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -574,7 +574,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>51.6</v>
+        <v>82.2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -583,17 +583,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="E3" t="n">
-        <v>154</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>779.2</v>
+        <v>1000</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -627,47 +627,47 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>OFRECE EN VENTA</t>
+          <t>DEPARTAMENTO 3 AMBIENTES EN VENTA EN 25 DE MAYO, MENDOZA CAPITAL</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/18739/ficha/casa-en-venta-en-montevideo-700</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19405/ficha/departamento-en-venta-en-25-de-mayo-900</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 100,000) | 🛡️ Cuenta con seguridad 24 hs / barrio privado | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>48.3</v>
+        <v>60.5</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>130000</v>
+        <v>140000</v>
       </c>
       <c r="E4" t="n">
-        <v>75</v>
+        <v>195</v>
       </c>
       <c r="F4" t="n">
-        <v>1733.3</v>
+        <v>717.9</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -701,17 +701,17 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>"CARINA DROZD gestiones inmobiliarias" VENDE: DEPARTAMENTOS Ubicadísimos: Calle ALMIRANTE BROWN, B° BOMBAL SUR. Complejo de 7 deptos con cocheras subterráneas. ASCENSOR. Piso 1 y Piso 2. FRONTALES!. Constan de: COCINA LIVING COMEDOR con Equipo A.A. y Calefactor; cocina con extractor, alacenas, bajomesada, Barra Desayunador- 2 DORMITORIOS (1 con A.A.) con Placares y Calefactores- 2 BAÑOS (uno en SUITE)- Recién Pintados! BALCON- PATIO LAVANDERÍA con bacha y mueble- COCHERA AUTOMATIZADA, en Subsuelo. VALORES: U$S 115.000 sin cochera en Piso 1- U$S 130.000 con Cochera en Piso 2. ESCRITURACION Inmediata. ALQUILADOS con Excelentes Rentas, pero se desocupan si lo desea el comprador-</t>
+          <t>Casa en venta en esquina – Dorrego, Guaymallén</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/1406-carina-drozd-gestiones-inmobiliarias/inmuebles/3601/ficha/departamento-en-venta-en-almirante-brown-1524</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19775/ficha/casa-en-venta-en-juan-b-justo-1200</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -722,11 +722,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>45.7</v>
+        <v>55.3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -735,17 +735,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>140000</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
+        <v>79000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>110</v>
+      </c>
+      <c r="F5" t="n">
+        <v>718.2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -754,7 +750,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -779,17 +775,17 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>OPENHOUSE VENDE | Exclusivos departamentos en pozo – Quinta Sección</t>
+          <t>Bombal Sur. Piso completo - Beltran 1.910 esquina 25 de Mayo. Excelente ubicacion geografica. Cerca Estacion Metrotanvia. Limite con Barrio Bombal de Ciudad. 2° Piso. Muy luminoso . Living comedor amplio. Cocina comedor mediana. 3 dormitorios con placares. 2 baños. Ascensor .Apto Credito . Desocupado. Javier / Armando</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2240/ficha/departamento-en-venta-en-5ta-seccion</t>
+          <t>https://www.inmoclick.com.ar/16797-provivienda-inmobiliaria/inmuebles/811/ficha/departamento-en-venta-en-beltran-1-910</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | ✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 79,000) | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -800,7 +796,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>45.3</v>
+        <v>50.3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -813,13 +809,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>79000</v>
+        <v>95000</v>
       </c>
       <c r="E6" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F6" t="n">
-        <v>718.2</v>
+        <v>871.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -828,7 +824,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -853,28 +849,28 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Bombal Sur. Piso completo - Beltran 1.910 esquina 25 de Mayo. Excelente ubicacion geografica. Cerca Estacion Metrotanvia. Limite con Barrio Bombal de Ciudad. 2° Piso. Muy luminoso . Living comedor amplio. Cocina comedor mediana. 3 dormitorios con placares. 2 baños. Ascensor .Apto Credito . Desocupado. Javier / Armando</t>
+          <t>VENTA DEPARTAMENTO – GODOY CRUZ</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/16797-provivienda-inmobiliaria/inmuebles/811/ficha/departamento-en-venta-en-beltran-1-910</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1974/ficha/departamento-en-venta-en-avenida-san-martin-100</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 79,000) | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>44.6</v>
+        <v>48.4</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -887,22 +883,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>90000</v>
+        <v>55000</v>
       </c>
       <c r="E7" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="F7" t="n">
-        <v>1384.6</v>
+        <v>763.9</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -927,28 +923,28 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Departamento ubicado en 5° piso de Avenida Pedro Molina, Segunda sección de Capital.</t>
+          <t>DEPARTAMENTO DE 4 AMBIENTES - CENTRICO</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/105122-helga-kruls-propiedades/inmuebles/121/ficha/departamento-en-venta-en-pedro-molina-461</t>
+          <t>https://www.inmoclick.com.ar/68264-gaustralinmobiliariaatgmail-com/inmuebles/4/ficha/departamento-en-venta-en-rondeau</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000) | 🔥 Red de gas natural confirmada</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>40.3</v>
+        <v>48.3</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -961,13 +957,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>95000</v>
+        <v>130000</v>
       </c>
       <c r="E8" t="n">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F8" t="n">
-        <v>871.6</v>
+        <v>1733.3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1001,28 +997,28 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>VENTA DEPARTAMENTO – GODOY CRUZ</t>
+          <t>"CARINA DROZD gestiones inmobiliarias" VENDE: DEPARTAMENTOS Ubicadísimos: Calle ALMIRANTE BROWN, B° BOMBAL SUR. Complejo de 7 deptos con cocheras subterráneas. ASCENSOR. Piso 1 y Piso 2. FRONTALES!. Constan de: COCINA LIVING COMEDOR con Equipo A.A. y Calefactor; cocina con extractor, alacenas, bajomesada, Barra Desayunador- 2 DORMITORIOS (1 con A.A.) con Placares y Calefactores- 2 BAÑOS (uno en SUITE)- Recién Pintados! BALCON- PATIO LAVANDERÍA con bacha y mueble- COCHERA AUTOMATIZADA, en Subsuelo. VALORES: U$S 115.000 sin cochera en Piso 1- U$S 130.000 con Cochera en Piso 2. ESCRITURACION Inmediata. ALQUILADOS con Excelentes Rentas, pero se desocupan si lo desea el comprador-</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1974/ficha/departamento-en-venta-en-avenida-san-martin-100</t>
+          <t>https://www.inmoclick.com.ar/1406-carina-drozd-gestiones-inmobiliarias/inmuebles/3601/ficha/departamento-en-venta-en-almirante-brown-1524</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>38.4</v>
+        <v>47.3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1035,17 +1031,17 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>55000</v>
+        <v>90000</v>
       </c>
       <c r="E9" t="n">
-        <v>72</v>
+        <v>137</v>
       </c>
       <c r="F9" t="n">
-        <v>763.9</v>
+        <v>656.9</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No/Duda</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1075,47 +1071,47 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO DE 4 AMBIENTES - CENTRICO</t>
+          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/68264-gaustralinmobiliariaatgmail-com/inmuebles/4/ficha/departamento-en-venta-en-rondeau</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 55,000) | 🔥 Red de gas natural confirmada</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000)</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>37.3</v>
+        <v>47.1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>90000</v>
+        <v>110000</v>
       </c>
       <c r="E10" t="n">
-        <v>137</v>
+        <v>191</v>
       </c>
       <c r="F10" t="n">
-        <v>656.9</v>
+        <v>575.9</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1124,7 +1120,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1149,32 +1145,32 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
+          <t>Venta casa 3 dormitorios con jardín y cochera – Dorrego, Guaymallén</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/20180/ficha/casa-en-venta-en-juan-jose-paso-1400</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 110,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>35.7</v>
+        <v>45.7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1183,13 +1179,17 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>55000</v>
-      </c>
-      <c r="E11" t="n">
-        <v>88</v>
-      </c>
-      <c r="F11" t="n">
-        <v>625</v>
+        <v>140000</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1223,17 +1223,17 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
+          <t>OPENHOUSE VENDE | Exclusivos departamentos en pozo – Quinta Sección</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
+          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2240/ficha/departamento-en-venta-en-5ta-seccion</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 55,000)</t>
+          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1244,7 +1244,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>35.3</v>
+        <v>45.7</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1257,13 +1257,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>110000</v>
+        <v>55000</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="F12" t="n">
-        <v>1100</v>
+        <v>625</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1297,17 +1297,17 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Departamento En Coronel Dorrego</t>
+          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 110,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1318,7 +1318,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>35.1</v>
+        <v>45.1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 70,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 70,000)</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1392,7 +1392,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>34.6</v>
+        <v>44.6</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 53,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 53,000)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1466,11 +1466,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>34</v>
+        <v>44.6</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>120000</v>
+        <v>90000</v>
       </c>
       <c r="E15" t="n">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="F15" t="n">
-        <v>1333.3</v>
+        <v>1384.6</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1519,17 +1519,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Departamento Premium De 2 Dormitorios 2 Baños Y Amenitis. En Dorrego Guaymallen</t>
+          <t>Departamento ubicado en 5° piso de Avenida Pedro Molina, Segunda sección de Capital.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2052069609-departamento-premium-de-2-dormitorios-2-banos-y-amenitis-en-dorrego-guaymallen-_JM</t>
+          <t>https://www.inmoclick.com.ar/105122-helga-kruls-propiedades/inmuebles/121/ficha/departamento-en-venta-en-pedro-molina-461</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 120,000)</t>
+          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1540,11 +1540,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>33.5</v>
+        <v>44</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1553,13 +1553,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>124900</v>
+        <v>120000</v>
       </c>
       <c r="E16" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F16" t="n">
-        <v>1435.6</v>
+        <v>1333.3</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1593,17 +1593,17 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Venta Hermoso Departamento Duplex - Barrio Bombal</t>
+          <t>Departamento Premium De 2 Dormitorios 2 Baños Y Amenitis. En Dorrego Guaymallen</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1945076259-venta-hermoso-departamento-duplex-barrio-bombal-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2052069609-departamento-premium-de-2-dormitorios-2-banos-y-amenitis-en-dorrego-guaymallen-_JM</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 124,900)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 120,000)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1614,7 +1614,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>33.1</v>
+        <v>43.5</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1627,13 +1627,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>75000</v>
+        <v>124900</v>
       </c>
       <c r="E17" t="n">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="F17" t="n">
-        <v>1000</v>
+        <v>1435.6</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1667,28 +1667,28 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
+          <t>Venta Hermoso Departamento Duplex - Barrio Bombal</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1945076259-venta-hermoso-departamento-duplex-barrio-bombal-_JM</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | ✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 124,900)</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>32.7</v>
+        <v>43.1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1701,13 +1701,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>86000</v>
+        <v>75000</v>
       </c>
       <c r="E18" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F18" t="n">
-        <v>1228.6</v>
+        <v>1000</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1741,17 +1741,17 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
+          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
+          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1762,11 +1762,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>30.2</v>
+        <v>35.3</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1775,13 +1775,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>140000</v>
+        <v>110000</v>
       </c>
       <c r="E19" t="n">
-        <v>575</v>
+        <v>100</v>
       </c>
       <c r="F19" t="n">
-        <v>243.5</v>
+        <v>1100</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1815,28 +1815,28 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>OPENHOUSE vende desarrollo en obra gruesa sobre calle Pascual Segura de Godoy Cruz</t>
+          <t>Departamento En Coronel Dorrego</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2063/ficha/departamento-en-venta-en-pascual-segura-godoy-cruz</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 110,000)</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>21.6</v>
+        <v>32.7</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1849,13 +1849,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>58000</v>
+        <v>86000</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F20" t="n">
-        <v>580</v>
+        <v>1228.6</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1889,17 +1889,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Duplex En Godoy Cruz</t>
+          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 58,000)</t>
+          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -1910,7 +1910,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20.9</v>
+        <v>31.6</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1923,13 +1923,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>80000</v>
+        <v>58000</v>
       </c>
       <c r="E21" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="F21" t="n">
-        <v>888.9</v>
+        <v>580</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1963,17 +1963,17 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
+          <t>Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 80,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 58,000)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -1984,7 +1984,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20.3</v>
+        <v>30.3</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 99,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 99,000)</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2058,7 +2058,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2132,7 +2132,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2145,13 +2145,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>86000</v>
+        <v>150000</v>
       </c>
       <c r="E24" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="F24" t="n">
-        <v>1211.3</v>
+        <v>1898.7</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2180,33 +2180,33 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Venta Departamento Godoy Cruz. Complejo Privado. Dto 11</t>
+          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1746780419-venta-departamento-godoy-cruz-complejo-privado-dto-11-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 86,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2219,13 +2219,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>63300</v>
+        <v>128000</v>
       </c>
       <c r="E25" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F25" t="n">
-        <v>867.1</v>
+        <v>1471.3</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2259,17 +2259,17 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Departamento En Gobernador Benegas</t>
+          <t>Venta Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 63,300)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 128,000)</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2280,7 +2280,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20</v>
+        <v>20.9</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2293,13 +2293,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>150000</v>
+        <v>80000</v>
       </c>
       <c r="E26" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="F26" t="n">
-        <v>1898.7</v>
+        <v>888.9</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2328,23 +2328,27 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Estándar</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
+          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr"/>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 80,000)</t>
+        </is>
+      </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
@@ -2363,13 +2367,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>128000</v>
+        <v>86000</v>
       </c>
       <c r="E27" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="F27" t="n">
-        <v>1471.3</v>
+        <v>1211.3</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2403,20 +2407,94 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Venta Duplex En Godoy Cruz</t>
+          <t>Venta Departamento Godoy Cruz. Complejo Privado. Dto 11</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1746780419-venta-departamento-godoy-cruz-complejo-privado-dto-11-_JM</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 128,000)</t>
+          <t>Dentro del presupuesto (USD 86,000)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>20</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>63300</v>
+      </c>
+      <c r="E28" t="n">
+        <v>73</v>
+      </c>
+      <c r="F28" t="n">
+        <v>867.1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Departamento En Gobernador Benegas</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 63,300)</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
         <is>
           <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>

</xml_diff>

<commit_message>
fix: filtro semantico negativo para descartar zonas excluidas explicitas (ej. Maipu/Luzuriaga)
</commit_message>
<xml_diff>
--- a/data/oportunidades_mendoza.xlsx
+++ b/data/oportunidades_mendoza.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,26 +796,26 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>47.8</v>
+        <v>47.3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>98000</v>
+        <v>90000</v>
       </c>
       <c r="E6" t="n">
-        <v>162</v>
+        <v>137</v>
       </c>
       <c r="F6" t="n">
-        <v>604.9</v>
+        <v>656.9</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -824,7 +824,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -844,37 +844,37 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Estándar</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>GYG Gestiones Inmobiliarias ofrece a la VENTA una amplia y funcional propiedad ubicada sobre calle Juan de Guevara, en Luzuriaga, Maipú – Mendoza.</t>
+          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/311068-gyg-gestiones-inmobiliarias/inmuebles/1/ficha/casa-en-venta-en-juan-de-guevara-3326</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 98,000) | 🚗 Cuenta con cochera | 💡 Publicación indica apertura a ofertas o permutas</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000)</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>47.3</v>
+        <v>45.7</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -883,13 +883,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>90000</v>
+        <v>55000</v>
       </c>
       <c r="E7" t="n">
-        <v>137</v>
+        <v>88</v>
       </c>
       <c r="F7" t="n">
-        <v>656.9</v>
+        <v>625</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -923,17 +923,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
+          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -944,11 +944,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>45.7</v>
+        <v>45.5</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -957,13 +957,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>55000</v>
+        <v>65000</v>
       </c>
       <c r="E8" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F8" t="n">
-        <v>625</v>
+        <v>764.7</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -997,17 +997,17 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
+          <t>RICCARDI PROPIEDADES VENDE espectacular departamento en Barrio Bombal Sur, Godoy Cruz, sobre calle Beltrán entre Tucumán y Juan B. Justo.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
+          <t>https://www.inmoclick.com.ar/3331-riccardi-propiedades/inmuebles/537/ficha/departamento-en-venta-en-beltran-1632-godoy-cruz-mendoza</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | ✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 65,000)</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1018,7 +1018,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1031,13 +1031,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>65000</v>
+        <v>124900</v>
       </c>
       <c r="E9" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F9" t="n">
-        <v>764.7</v>
+        <v>1435.6</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1071,17 +1071,17 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>RICCARDI PROPIEDADES VENDE espectacular departamento en Barrio Bombal Sur, Godoy Cruz, sobre calle Beltrán entre Tucumán y Juan B. Justo.</t>
+          <t>Venta Hermoso Departamento Duplex - Barrio Bombal</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/3331-riccardi-propiedades/inmuebles/537/ficha/departamento-en-venta-en-beltran-1632-godoy-cruz-mendoza</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1945076259-venta-hermoso-departamento-duplex-barrio-bombal-_JM</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | ✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 65,000)</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | ✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 124,900)</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1092,11 +1092,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>43.5</v>
+        <v>43.1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1105,13 +1105,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>124900</v>
+        <v>75000</v>
       </c>
       <c r="E10" t="n">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="F10" t="n">
-        <v>1435.6</v>
+        <v>1000</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1145,32 +1145,32 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Venta Hermoso Departamento Duplex - Barrio Bombal</t>
+          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1945076259-venta-hermoso-departamento-duplex-barrio-bombal-_JM</t>
+          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | ✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 124,900)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>43.1</v>
+        <v>35.3</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>75000</v>
+        <v>110000</v>
       </c>
       <c r="E11" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="F11" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1219,32 +1219,32 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO ubicado en Torres San Vicente sobre calle San Martín Sur 499 frente calle Leguizamón - Godoy Cruz - Mendoza.</t>
+          <t>Departamento En Coronel Dorrego</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/754/ficha/departamento-en-venta-en-torres-san-vicente-godoy-cruz-mendoza</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 75,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 110,000)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>35.3</v>
+        <v>32.7</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1253,13 +1253,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>110000</v>
+        <v>86000</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F12" t="n">
-        <v>1100</v>
+        <v>1228.6</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1293,28 +1293,28 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Departamento En Coronel Dorrego</t>
+          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 110,000)</t>
+          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>32.7</v>
+        <v>31.6</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1327,13 +1327,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>86000</v>
+        <v>58000</v>
       </c>
       <c r="E13" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F13" t="n">
-        <v>1228.6</v>
+        <v>580</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1367,17 +1367,17 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Oportunidad! Venta Departamento Godoy Cruz - 2 dormitorios, con cochera subterránea y ascensor</t>
+          <t>Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/1981/ficha/departamento-en-venta-en-belgrano-200</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 86,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 58,000)</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1388,7 +1388,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>31.6</v>
+        <v>30.3</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>58000</v>
+        <v>99000</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F14" t="n">
-        <v>580</v>
+        <v>1064.5</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1441,17 +1441,17 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Duplex En Godoy Cruz</t>
+          <t>Venta Amplio Departamento Godoy Cruz  Apto Credito</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3912396714-venta-amplio-departamento-godoy-cruz-apto-credito-_JM</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 58,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 99,000)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1462,7 +1462,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>30.3</v>
+        <v>30</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1475,13 +1475,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>99000</v>
+        <v>150000</v>
       </c>
       <c r="E15" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="F15" t="n">
-        <v>1064.5</v>
+        <v>2027</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1510,27 +1510,27 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Venta Amplio Departamento Godoy Cruz  Apto Credito</t>
+          <t>Venta Departamento Godoy Cruz Con Cochera</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3912396714-venta-amplio-departamento-godoy-cruz-apto-credito-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1805521295-venta-departamento-godoy-cruz-con-cochera-_JM</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 99,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
@@ -1552,10 +1552,10 @@
         <v>150000</v>
       </c>
       <c r="E16" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F16" t="n">
-        <v>2027</v>
+        <v>1898.7</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1589,17 +1589,17 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Venta Departamento Godoy Cruz Con Cochera</t>
+          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1805521295-venta-departamento-godoy-cruz-con-cochera-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>150000</v>
+        <v>128000</v>
       </c>
       <c r="E17" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F17" t="n">
-        <v>1898.7</v>
+        <v>1471.3</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1658,33 +1658,33 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Estándar</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
+          <t>Venta Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 128,000)</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>30</v>
+        <v>20.9</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1697,13 +1697,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>128000</v>
+        <v>80000</v>
       </c>
       <c r="E18" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F18" t="n">
-        <v>1471.3</v>
+        <v>888.9</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1737,17 +1737,17 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Venta Duplex En Godoy Cruz</t>
+          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 128,000)</t>
+          <t>Dentro del presupuesto (USD 80,000)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1758,7 +1758,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>20.9</v>
+        <v>20.6</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1774,10 +1774,10 @@
         <v>80000</v>
       </c>
       <c r="E19" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F19" t="n">
-        <v>888.9</v>
+        <v>930.2</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
+          <t>Dúplex En Venta -g.cruz-id:314510</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3724250208-duplex-en-venta-gcruz-id314510-_JM</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1832,7 +1832,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>20.6</v>
+        <v>20</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1845,13 +1845,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>80000</v>
+        <v>63300</v>
       </c>
       <c r="E20" t="n">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="F20" t="n">
-        <v>930.2</v>
+        <v>867.1</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1885,94 +1885,20 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Dúplex En Venta -g.cruz-id:314510</t>
+          <t>Departamento En Gobernador Benegas</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3724250208-duplex-en-venta-gcruz-id314510-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 80,000)</t>
+          <t>Dentro del presupuesto (USD 63,300)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
-        <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>63300</v>
-      </c>
-      <c r="E21" t="n">
-        <v>73</v>
-      </c>
-      <c r="F21" t="n">
-        <v>867.1</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Departamento En Gobernador Benegas</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 63,300)</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
         <is>
           <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>

</xml_diff>

<commit_message>
fix: corregir parseo de features en argenprop y sincronizar datos locales
</commit_message>
<xml_diff>
--- a/data/oportunidades_mendoza.xlsx
+++ b/data/oportunidades_mendoza.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>66.2</v>
+        <v>63.5</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -509,17 +509,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>63000</v>
+        <v>80000</v>
       </c>
       <c r="E2" t="n">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="F2" t="n">
-        <v>463.2</v>
+        <v>666.7</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -553,17 +553,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>OPORTUNIDAD EN PLENO CENTRO</t>
+          <t>CASA EN IMPORTANTE ESQUINA DE LA CIUDAD.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/133635-di-luca-propiedades/inmuebles/102/ficha/departamento-en-venta-en-buenos-aires-n0-258-ciudad</t>
+          <t>https://www.inmoclick.com.ar/136928-amtpropiedades/inmuebles/10/ficha/casa-en-venta-en-chile-y-coronel-plaza</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 80,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -574,7 +574,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>63.5</v>
+        <v>62.9</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -587,13 +587,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>85000</v>
+        <v>95000</v>
       </c>
       <c r="E3" t="n">
-        <v>129</v>
+        <v>294</v>
       </c>
       <c r="F3" t="n">
-        <v>658.9</v>
+        <v>323.1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -627,17 +627,17 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>En la hermosa ciudad de Mendoza, en la 6.ª Sección Residencial Norte, se encuentra esta propiedad ideal para aquellos que buscan invertir en un proyecto de reciclaje o construcción de departamentos. La casa, de 50 años de antigüedad, se encuentra totalmente construida en material y cuenta con un lote de 10 x 25.50 metros.</t>
+          <t>Re/Max Terruños ofrece a la venta propiedad ubicada en esquina, de construcción mixta, con 300 m² cubiertos aproximadamente, ideal tanto para vivienda familiar como para actividades profesionales.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/298285-pablo-catalano/inmuebles/3/ficha/casa-en-venta-en-maure-250</t>
+          <t>https://www.inmoclick.com.ar/229229-remax-terrunos/inmuebles/2778/ficha/casa-en-venta-en-espana-2900</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 85,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -648,7 +648,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>62.9</v>
+        <v>62.2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -661,13 +661,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>95000</v>
+        <v>88000</v>
       </c>
       <c r="E4" t="n">
-        <v>294</v>
+        <v>99</v>
       </c>
       <c r="F4" t="n">
-        <v>323.1</v>
+        <v>888.9</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -701,17 +701,17 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Re/Max Terruños ofrece a la venta propiedad ubicada en esquina, de construcción mixta, con 300 m² cubiertos aproximadamente, ideal tanto para vivienda familiar como para actividades profesionales.</t>
+          <t>CASA EN VENTA 3 DORMITORIOS 2 BAÑOS SOBERANÍA NACIONAL MENDOZA - APTO CRÉDITO</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/229229-remax-terrunos/inmuebles/2778/ficha/casa-en-venta-en-espana-2900</t>
+          <t>https://www.inmoclick.com.ar/229229-remax-terrunos/inmuebles/2593/ficha/casa-en-venta-en-posta-retamo-0</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 88,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -722,7 +722,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>62.8</v>
+        <v>51.5</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -731,21 +731,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>98000</v>
+        <v>125000</v>
       </c>
       <c r="E5" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="F5" t="n">
-        <v>490</v>
+        <v>1562.5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -770,33 +770,33 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>CASA EN VENTA</t>
+          <t>COCUCCI INMOBILIARIA VENDE Exclusivo departamento de categoría en el prestigioso Barrio Bombal – Godoy Cruz</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/29719-martin-helder/inmuebles/52/ficha/casa-en-venta-en-beltran-425</t>
+          <t>https://www.inmoclick.com.ar/17-cocucci-sa/inmuebles/20148/ficha/departamento-en-venta-en-arizu-al-278</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 98,000) | 🚗 Cuenta con cochera</t>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 125,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>62.2</v>
+        <v>50.8</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -805,21 +805,21 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>88000</v>
+        <v>68000</v>
       </c>
       <c r="E6" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>888.9</v>
+        <v>906.7</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -849,28 +849,28 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>CASA EN VENTA 3 DORMITORIOS 2 BAÑOS SOBERANÍA NACIONAL MENDOZA - APTO CRÉDITO</t>
+          <t>DRUMMOND NEGOCIOS INMOBILIARIOS VENDE</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/229229-remax-terrunos/inmuebles/2593/ficha/casa-en-venta-en-posta-retamo-0</t>
+          <t>https://www.inmoclick.com.ar/124071-drummond-negocios-inmobiliarios/inmuebles/43/ficha/departamento-en-venta-en-espana-y-gutierrez</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 88,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 68,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>62.1</v>
+        <v>49.9</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -879,17 +879,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Departamento</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>110000</v>
+        <v>70000</v>
       </c>
       <c r="E7" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="F7" t="n">
-        <v>687.5</v>
+        <v>1000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -923,17 +923,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ofrece una excelente propiedad en una ubicación estratégica a minutos del parque san martín , centros de salud , colegios.</t>
+          <t>Venta de Departamento – Cuarta Sección Oeste</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/20387/ficha/casa-en-venta-en-huarpes-1800</t>
+          <t>https://www.inmoclick.com.ar/3076-ente-inmobiliaria/inmuebles/3329/ficha/departamento-en-venta-en-fray-inalican-363</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 110,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 70,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -944,7 +944,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>53.4</v>
+        <v>48.8</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -957,17 +957,17 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>95000</v>
+        <v>129000</v>
       </c>
       <c r="E8" t="n">
-        <v>77</v>
+        <v>114</v>
       </c>
       <c r="F8" t="n">
-        <v>1233.8</v>
+        <v>1131.6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -997,28 +997,28 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Departamento ubicado en una zona estratégica, a poca distancia de Plaza Independencia: una propuesta ideal para quienes buscan comodidad y funcionalidad en el centro. Se trata de un 1° piso frontal que ofrece ambientes bien distribuidos y posibilidades para adaptarlo según tus necesidades.</t>
+          <t>DEPARTAMENTO 9 AMBIENTES EN VENTA - GODOY CRUZ - MENDOZA - 157 M²</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/11968-inmobiliaria-miguel-angel-juan-pablo-simon/inmuebles/51/ficha/departamento-en-venta-en-gutierrez-434</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/18971/ficha/departamento-en-venta-en-juan-de-garay-400</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 129,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>51.5</v>
+        <v>47.3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1031,22 +1031,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>125000</v>
+        <v>90000</v>
       </c>
       <c r="E9" t="n">
-        <v>80</v>
+        <v>137</v>
       </c>
       <c r="F9" t="n">
-        <v>1562.5</v>
+        <v>656.9</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No/Duda</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1066,33 +1066,33 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Estándar</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>COCUCCI INMOBILIARIA VENDE Exclusivo departamento de categoría en el prestigioso Barrio Bombal – Godoy Cruz</t>
+          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17-cocucci-sa/inmuebles/20148/ficha/departamento-en-venta-en-arizu-al-278</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | Dentro del presupuesto (USD 125,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000)</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>50.8</v>
+        <v>46.8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1105,17 +1105,17 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>68000</v>
+        <v>105000</v>
       </c>
       <c r="E10" t="n">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="F10" t="n">
-        <v>906.7</v>
+        <v>954.5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No/Duda</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1145,32 +1145,32 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>DRUMMOND NEGOCIOS INMOBILIARIOS VENDE</t>
+          <t>Departamento en venta , Calle Gutierrez, Ciudad de Mendoza . Amoblado.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/124071-drummond-negocios-inmobiliarios/inmuebles/43/ficha/departamento-en-venta-en-espana-y-gutierrez</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19925/ficha/departamento-en-venta-en-gutierrez-400</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 68,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 105,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>48.8</v>
+        <v>45.7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>129000</v>
+        <v>55000</v>
       </c>
       <c r="E11" t="n">
-        <v>114</v>
+        <v>88</v>
       </c>
       <c r="F11" t="n">
-        <v>1131.6</v>
+        <v>625</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No/Duda</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1219,28 +1219,28 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO 9 AMBIENTES EN VENTA - GODOY CRUZ - MENDOZA - 157 M²</t>
+          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/18971/ficha/departamento-en-venta-en-juan-de-garay-400</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 129,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>47.3</v>
+        <v>45</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1256,10 +1256,10 @@
         <v>90000</v>
       </c>
       <c r="E12" t="n">
-        <v>137</v>
+        <v>82</v>
       </c>
       <c r="F12" t="n">
-        <v>656.9</v>
+        <v>1097.6</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
+          <t>Vendo Departamento en Ciudad de Mendoza. 82 mtrs terreno total. La propiedad cuenta con cocina comedor, living, 3 habitaciones, placares, 2 baños, aire acondicionado, calefactores. Los principales ventanales dan a la cordillera. En pleno centro de Mendoza. Se evalúan ofertas. Zelta Inmobiliaria</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
+          <t>https://www.inmoclick.com.ar/302127-zelta-inmobiliaria/inmuebles/95/ficha/departamento-en-venta-en-catamarca-35</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1314,7 +1314,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>46.8</v>
+        <v>44.9</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1327,13 +1327,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>105000</v>
+        <v>77500</v>
       </c>
       <c r="E13" t="n">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="F13" t="n">
-        <v>954.5</v>
+        <v>1174.2</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1367,17 +1367,17 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Departamento en venta , Calle Gutierrez, Ciudad de Mendoza . Amoblado.</t>
+          <t>Follow ofrece en venta un amplio departamento de 3 dormitorios, totalmente refaccionado, ubicado sobre calle Amigorena, en pleno centro de la Ciudad de Mendoza.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/19925/ficha/departamento-en-venta-en-gutierrez-400</t>
+          <t>https://www.inmoclick.com.ar/274909-remax-follow/inmuebles/2357/ficha/departamento-en-venta-en-amigorena-0</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 105,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 77,500) | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1388,11 +1388,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>45.7</v>
+        <v>41.9</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>55000</v>
+        <v>68000</v>
       </c>
       <c r="E14" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F14" t="n">
-        <v>625</v>
+        <v>708.3</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1441,32 +1441,32 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
+          <t>SILVIA NAPOLI CORREDORA PUBLICA MAT 724, vende departamento en Coronel Dorrego, Guaymallén, Mendoza. Ubicación privilegiada.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
+          <t>https://www.inmoclick.com.ar/251492-silvia-napoli/inmuebles/197/ficha/departamento-en-venta-en-joaquin-v-gonzalez-325</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 68,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>45</v>
+        <v>35.3</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1475,13 +1475,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>90000</v>
+        <v>110000</v>
       </c>
       <c r="E15" t="n">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>1097.6</v>
+        <v>1100</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1515,17 +1515,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Vendo Departamento en Ciudad de Mendoza. 82 mtrs terreno total. La propiedad cuenta con cocina comedor, living, 3 habitaciones, placares, 2 baños, aire acondicionado, calefactores. Los principales ventanales dan a la cordillera. En pleno centro de Mendoza. Se evalúan ofertas. Zelta Inmobiliaria</t>
+          <t>Departamento En Coronel Dorrego</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/302127-zelta-inmobiliaria/inmuebles/95/ficha/departamento-en-venta-en-catamarca-35</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000)</t>
+          <t>Dentro del presupuesto (USD 110,000)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1536,7 +1536,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>44.9</v>
+        <v>33.1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1549,13 +1549,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>77500</v>
+        <v>63000</v>
       </c>
       <c r="E16" t="n">
-        <v>66</v>
+        <v>112</v>
       </c>
       <c r="F16" t="n">
-        <v>1174.2</v>
+        <v>562.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1589,28 +1589,28 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Follow ofrece en venta un amplio departamento de 3 dormitorios, totalmente refaccionado, ubicado sobre calle Amigorena, en pleno centro de la Ciudad de Mendoza.</t>
+          <t>Oportunidad de inversión!</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/274909-remax-follow/inmuebles/2357/ficha/departamento-en-venta-en-amigorena-0</t>
+          <t>https://www.inmoclick.com.ar/259304-bcg-desarrollos-inmobiliarios/inmuebles/28/ficha/departamento-en-venta-en-pte-derqui-243</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 77,500) | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>41.9</v>
+        <v>31.6</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>68000</v>
+        <v>58000</v>
       </c>
       <c r="E17" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F17" t="n">
-        <v>708.3</v>
+        <v>580</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1663,17 +1663,17 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>SILVIA NAPOLI CORREDORA PUBLICA MAT 724, vende departamento en Coronel Dorrego, Guaymallén, Mendoza. Ubicación privilegiada.</t>
+          <t>Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/251492-silvia-napoli/inmuebles/197/ficha/departamento-en-venta-en-joaquin-v-gonzalez-325</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 68,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 58,000)</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1684,11 +1684,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>39.8</v>
+        <v>30.7</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1697,13 +1697,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>130000</v>
+        <v>55000</v>
       </c>
       <c r="E18" t="n">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="F18" t="n">
-        <v>1756.8</v>
+        <v>625</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1737,32 +1737,32 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>TRE INMOBILIARIA VENDE DEPARTAMENTO  ubicado sobre calle Huarpes 2046 - Sexta Sección - Mendoza.</t>
+          <t>DEPARTAMENTO EN VENTA CON BALCÓN EN CORONEL DORREGO, GUAYMALLÉN, MENDOZA</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/12572-tre-inmobiliaria/inmuebles/844/ficha/departamento-en-venta-en-sexta-seccion-ciudad-mendoza</t>
+          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/2417/ficha/departamento-en-venta-en-falucho-300</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 130,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>35.3</v>
+        <v>30</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1771,13 +1771,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>110000</v>
+        <v>53000</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F19" t="n">
-        <v>1100</v>
+        <v>757.1</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1811,28 +1811,28 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Departamento En Coronel Dorrego</t>
+          <t>Planta baja confortable y funcional en excelente zona de Dorrego, entre las calles Laprida y Cobos, adyacencias calle Lamadrid, ideal para quienes buscan comodidad, privacidad y ubicación estratégica. Un hogar pensado para el día a día: living comedor para recibir visitas, cocina comedor práctica para las comidas diarias y una lavandería independiente que facilita las tareas del hogar. Tres dormitorios bien distribuidos: dos con placares y un tercero en suite con su propio placard, que ofrece mayor privacidad y confort.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
+          <t>https://www.inmoclick.com.ar/308706-cm/inmuebles/6/ficha/departamento-en-venta-en-laprida-y-cobos</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 110,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 53,000)</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>31.6</v>
+        <v>30</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1845,13 +1845,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>58000</v>
+        <v>150000</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="F20" t="n">
-        <v>580</v>
+        <v>1898.7</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1880,33 +1880,33 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Duplex En Godoy Cruz</t>
+          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 58,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>30.7</v>
+        <v>30</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1919,13 +1919,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>55000</v>
+        <v>128000</v>
       </c>
       <c r="E21" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F21" t="n">
-        <v>625</v>
+        <v>1471.3</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1959,17 +1959,17 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO EN VENTA CON BALCÓN EN CORONEL DORREGO, GUAYMALLÉN, MENDOZA</t>
+          <t>Venta Duplex En Godoy Cruz</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/268429-re-max-vendimia/inmuebles/2417/ficha/departamento-en-venta-en-falucho-300</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 128,000)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -1980,7 +1980,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>30</v>
+        <v>20.9</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1993,13 +1993,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>53000</v>
+        <v>80000</v>
       </c>
       <c r="E22" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F22" t="n">
-        <v>757.1</v>
+        <v>888.9</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2033,17 +2033,17 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Planta baja confortable y funcional en excelente zona de Dorrego, entre las calles Laprida y Cobos, adyacencias calle Lamadrid, ideal para quienes buscan comodidad, privacidad y ubicación estratégica. Un hogar pensado para el día a día: living comedor para recibir visitas, cocina comedor práctica para las comidas diarias y una lavandería independiente que facilita las tareas del hogar. Tres dormitorios bien distribuidos: dos con placares y un tercero en suite con su propio placard, que ofrece mayor privacidad y confort.</t>
+          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/308706-cm/inmuebles/6/ficha/departamento-en-venta-en-laprida-y-cobos</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 53,000)</t>
+          <t>Dentro del presupuesto (USD 80,000)</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2054,7 +2054,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2067,13 +2067,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>150000</v>
+        <v>75000</v>
       </c>
       <c r="E23" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F23" t="n">
-        <v>1898.7</v>
+        <v>1119.4</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2102,33 +2102,33 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Estándar</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
+          <t>Departamento En Las Tortugas</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2133562131-departamento-en-las-tortugas-_JM</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts)</t>
+          <t>Dentro del presupuesto (USD 75,000)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2141,13 +2141,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>128000</v>
+        <v>63300</v>
       </c>
       <c r="E24" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="F24" t="n">
-        <v>1471.3</v>
+        <v>867.1</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2181,242 +2181,20 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Venta Duplex En Godoy Cruz</t>
+          <t>Departamento En Gobernador Benegas</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3914417650-venta-duplex-en-godoy-cruz-_JM</t>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 128,000)</t>
+          <t>Dentro del presupuesto (USD 63,300)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
-        <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>80000</v>
-      </c>
-      <c r="E25" t="n">
-        <v>90</v>
-      </c>
-      <c r="F25" t="n">
-        <v>888.9</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 80,000)</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>20</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>75000</v>
-      </c>
-      <c r="E26" t="n">
-        <v>67</v>
-      </c>
-      <c r="F26" t="n">
-        <v>1119.4</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>Departamento En Las Tortugas</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2133562131-departamento-en-las-tortugas-_JM</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 75,000)</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>20</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Godoy Cruz</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Departamento</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>63300</v>
-      </c>
-      <c r="E27" t="n">
-        <v>73</v>
-      </c>
-      <c r="F27" t="n">
-        <v>867.1</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>Departamento En Gobernador Benegas</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Dentro del presupuesto (USD 63,300)</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
         <is>
           <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>

</xml_diff>

<commit_message>
feat: reducir score minimo a 60 y registrar avisos enviados por whatsapp
</commit_message>
<xml_diff>
--- a/data/oportunidades_mendoza.xlsx
+++ b/data/oportunidades_mendoza.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>63.5</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -513,17 +513,17 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>80000</v>
+        <v>95000</v>
       </c>
       <c r="E2" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F2" t="n">
-        <v>666.7</v>
+        <v>730.8</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,28 +553,28 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>CASA EN IMPORTANTE ESQUINA DE LA CIUDAD.</t>
+          <t>Casa en venta c/ cochera en 6.ª sección residencial norte</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/136928-amtpropiedades/inmuebles/10/ficha/casa-en-venta-en-chile-y-coronel-plaza</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-seccion-6-residencial-norte-5-ambientes--19590149</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 80,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>62.8</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -587,17 +587,17 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>98000</v>
+        <v>120000</v>
       </c>
       <c r="E3" t="n">
-        <v>200</v>
+        <v>148</v>
       </c>
       <c r="F3" t="n">
-        <v>490</v>
+        <v>810.8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -627,32 +627,32 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>CASA EN VENTA</t>
+          <t>Casa en venta 3 dormitorios – jardín con churrasquera – 2 cocheras – sexta sección</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/29719-martin-helder/inmuebles/52/ficha/casa-en-venta-en-beltran-425</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-sexta-seccion-5-ambientes--20476730</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 98,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 120,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>62.1</v>
+        <v>69</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -661,13 +661,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>110000</v>
+        <v>65000</v>
       </c>
       <c r="E4" t="n">
-        <v>160</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
-        <v>687.5</v>
+        <v>866.7</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -701,32 +701,32 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ofrece una excelente propiedad en una ubicación estratégica a minutos del parque san martín , centros de salud , colegios.</t>
+          <t>Dúplex en venta c/ cochera en godoy cruz</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/20387/ficha/casa-en-venta-en-huarpes-1800</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-godoy-cruz-3-ambientes--19590152</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 110,000) | 🚗 Cuenta con cochera</t>
+          <t>Dentro del presupuesto (USD 65,000) | 🛡️ Cuenta con seguridad 24 hs / barrio privado | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>51.2</v>
+        <v>65.8</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -735,13 +735,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>63000</v>
+        <v>65000</v>
       </c>
       <c r="E5" t="n">
-        <v>136</v>
+        <v>108</v>
       </c>
       <c r="F5" t="n">
-        <v>463.2</v>
+        <v>601.9</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -775,28 +775,28 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>OPORTUNIDAD EN PLENO CENTRO</t>
+          <t>Departamento con terraza y quincho 106m2 ciudad mendoza</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/133635-di-luca-propiedades/inmuebles/102/ficha/departamento-en-venta-en-buenos-aires-n0-258-ciudad</t>
+          <t>https://www.argenprop.com/departamento-en-venta-en-mendoza-4-ambientes--19928492</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 63,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 65,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>47.3</v>
+        <v>63.5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -805,17 +805,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>90000</v>
+        <v>80000</v>
       </c>
       <c r="E6" t="n">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="F6" t="n">
-        <v>656.9</v>
+        <v>666.7</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -824,7 +824,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
+          <t>CASA EN IMPORTANTE ESQUINA DE LA CIUDAD.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
+          <t>https://www.inmoclick.com.ar/136928-amtpropiedades/inmuebles/10/ficha/casa-en-venta-en-chile-y-coronel-plaza</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 80,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -870,26 +870,26 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>46.6</v>
+        <v>62.9</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>120000</v>
+        <v>95000</v>
       </c>
       <c r="E7" t="n">
-        <v>150</v>
+        <v>294</v>
       </c>
       <c r="F7" t="n">
-        <v>800</v>
+        <v>323.1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -923,28 +923,28 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>🏢 DEPARTAMENTO EN VENTA – CAPITAL, MENDOZA</t>
+          <t>Re/Max Terruños ofrece a la venta propiedad ubicada en esquina, de construcción mixta, con 300 m² cubiertos aproximadamente, ideal tanto para vivienda familiar como para actividades profesionales.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/312047-alvarez-asociados/inmuebles/12/ficha/departamento-en-venta-en-olascoaga-n-o-1566-entre-agustin-alvarez-y-avellaneda</t>
+          <t>https://www.inmoclick.com.ar/229229-remax-terrunos/inmuebles/2778/ficha/casa-en-venta-en-espana-2900</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>45.7</v>
+        <v>62.9</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -953,21 +953,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>140000</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>N/D</t>
-        </is>
+        <v>95000</v>
+      </c>
+      <c r="E8" t="n">
+        <v>250</v>
+      </c>
+      <c r="F8" t="n">
+        <v>380</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1001,17 +997,17 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>OPENHOUSE VENDE | Exclusivos departamentos en pozo – Quinta Sección</t>
+          <t>Vendo casa en ciudad de mendoza. apta credito hipotecario</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/280057-openhouse-inmobiliaria/inmuebles/2240/ficha/departamento-en-venta-en-5ta-seccion</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-mendoza-7-ambientes--20386270</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1022,26 +1018,26 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>45.7</v>
+        <v>62.8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>55000</v>
+        <v>98000</v>
       </c>
       <c r="E9" t="n">
-        <v>88</v>
+        <v>200</v>
       </c>
       <c r="F9" t="n">
-        <v>625</v>
+        <v>490</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1050,7 +1046,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1075,17 +1071,17 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
+          <t>CASA EN VENTA</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
+          <t>https://www.inmoclick.com.ar/29719-martin-helder/inmuebles/52/ficha/casa-en-venta-en-beltran-425</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 98,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1096,7 +1092,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>45.1</v>
+        <v>62.8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1109,13 +1105,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>70000</v>
+        <v>98000</v>
       </c>
       <c r="E10" t="n">
-        <v>80</v>
+        <v>395</v>
       </c>
       <c r="F10" t="n">
-        <v>875</v>
+        <v>248.1</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1124,7 +1120,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1149,17 +1145,17 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>📍 En pleno corazón de la ciudad de Mendoza, este amplio departamento amoblado ofrece comodidad y practicidad en una ubicación difícil de igualar. Espacios bien distribuidos que invitan a sentirse en casa desde el primer momento: cocina funcional, estar-comedor acogedor y dos dormitorios que garantizan privacidad. El mobiliario incluido —camas, mesas de luz, comedor y sala con TV— permite mudarse sin preocupaciones, y la opción de alquiler sin muebles brinda flexibilidad según tus necesidades.</t>
+          <t>Complejo de 4 unidades. duplex + 3 departamentos a reciclar</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/311442-plus-valor/inmuebles/2/ficha/departamento-en-venta-en-9-de-julio-1570</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-mendoza-10-ambientes--20608486</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 70,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 98,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1170,7 +1166,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>44.6</v>
+        <v>62.7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1179,17 +1175,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>53000</v>
+        <v>100000</v>
       </c>
       <c r="E11" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="F11" t="n">
-        <v>757.1</v>
+        <v>500</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1198,7 +1194,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1223,17 +1219,17 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Planta baja confortable y funcional en excelente zona de Dorrego, entre las calles Laprida y Cobos, adyacencias calle Lamadrid, ideal para quienes buscan comodidad, privacidad y ubicación estratégica. Un hogar pensado para el día a día: living comedor para recibir visitas, cocina comedor práctica para las comidas diarias y una lavandería independiente que facilita las tareas del hogar. Tres dormitorios bien distribuidos: dos con placares y un tercero en suite con su propio placard, que ofrece mayor privacidad y confort.</t>
+          <t>Hauser vende casa interna</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/308706-cm/inmuebles/6/ficha/departamento-en-venta-en-laprida-y-cobos</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-quinta-seccion--19148242</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 53,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 100,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1244,7 +1240,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>44.6</v>
+        <v>62.1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1253,17 +1249,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>90000</v>
+        <v>110000</v>
       </c>
       <c r="E12" t="n">
-        <v>65</v>
+        <v>160</v>
       </c>
       <c r="F12" t="n">
-        <v>1384.6</v>
+        <v>687.5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1297,17 +1293,17 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Departamento ubicado en 5° piso de Avenida Pedro Molina, Segunda sección de Capital.</t>
+          <t>ofrece una excelente propiedad en una ubicación estratégica a minutos del parque san martín , centros de salud , colegios.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/105122-helga-kruls-propiedades/inmuebles/121/ficha/departamento-en-venta-en-pedro-molina-461</t>
+          <t>https://www.inmoclick.com.ar/17515-remax-solutions/inmuebles/20387/ficha/casa-en-venta-en-huarpes-1800</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 110,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1318,26 +1314,26 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>43</v>
+        <v>62.1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>89000</v>
+        <v>110000</v>
       </c>
       <c r="E13" t="n">
-        <v>118</v>
+        <v>185</v>
       </c>
       <c r="F13" t="n">
-        <v>754.2</v>
+        <v>594.6</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1371,47 +1367,47 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>SIGILO DESARROLLOS INMOBILIARIOS VENDE</t>
+          <t>Venta - casa en dorrego - 3 dormitorios   estudio / 2 baños</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/29891-sigilo-desarrollos-inmobiliarios/inmuebles/109/ficha/departamento-en-venta-en-paraguay-y-castelar</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-coronel-dorrego-7-ambientes--20364060</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 89,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 110,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>42.1</v>
+        <v>61.6</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>87500</v>
+        <v>120000</v>
       </c>
       <c r="E14" t="n">
-        <v>100</v>
+        <v>234</v>
       </c>
       <c r="F14" t="n">
-        <v>875</v>
+        <v>512.8</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1445,47 +1441,47 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>CORDON &amp; ASOCIADOS VENDE</t>
+          <t>Vendo casa en dorrego</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/27015-cordon-asociados/inmuebles/7/ficha/departamento-en-venta-en-san-martin-y-peatonal</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-coronel-dorrego-4-ambientes--19123113</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 87,500) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>42</v>
+        <v>60.6</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>77000</v>
+        <v>138000</v>
       </c>
       <c r="E15" t="n">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="F15" t="n">
-        <v>793.8</v>
+        <v>1150</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1519,56 +1515,56 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>VENTA DE DEPARTAMENTO DE 3 HABITACIONES CON TERRAZA PROPIA A RECICLAR A METROS DE LA PLAZA ITALIA, MENDOZA.</t>
+          <t>Casa en venta c/ cochera en 6.ª sección residencial norte</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/310522-ana-lucia-raina-propiedades/inmuebles/9/ficha/departamento-en-venta-en-peru-y-montevideo</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-seccion-6-residencial-norte-6-ambientes--19590925</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 77,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 138,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>39.2</v>
+        <v>58.6</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>110000</v>
+        <v>138000</v>
       </c>
       <c r="E16" t="n">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="F16" t="n">
-        <v>940.2</v>
+        <v>985.7</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1593,32 +1589,32 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>ZELTA Inmobiliaria Vendo Departamento en Ciudad de Mendoza.</t>
+          <t>Dúplex en venta c/ cochera en centro</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/302127-zelta-inmobiliaria/inmuebles/170/ficha/departamento-en-venta-en-general-paz-135</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-mendoza-3-ambientes--19590175</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 110,000) | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 138,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>38.4</v>
+        <v>58.1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1627,13 +1623,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>95000</v>
+        <v>87000</v>
       </c>
       <c r="E17" t="n">
-        <v>77</v>
+        <v>150</v>
       </c>
       <c r="F17" t="n">
-        <v>1233.8</v>
+        <v>580</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1667,32 +1663,32 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Departamento ubicado en una zona estratégica, a poca distancia de Plaza Independencia: una propuesta ideal para quienes buscan comodidad y funcionalidad en el centro. Se trata de un 1° piso frontal que ofrece ambientes bien distribuidos y posibilidades para adaptarlo según tus necesidades.</t>
+          <t>Depto venta cuarta oeste 3 dorm</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/11968-inmobiliaria-miguel-angel-juan-pablo-simon/inmuebles/51/ficha/departamento-en-venta-en-gutierrez-434</t>
+          <t>https://www.argenprop.com/departamento-en-venta-en-cuarta-seccion-6-ambientes--17673475</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 95,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 87,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>35.3</v>
+        <v>55.7</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Guaymallen</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1701,13 +1697,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>110000</v>
+        <v>84500</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F18" t="n">
-        <v>1100</v>
+        <v>1056.2</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1716,7 +1712,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1741,17 +1737,17 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Departamento En Coronel Dorrego</t>
+          <t>Departamento céntrico, calle 9 de julio</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
+          <t>https://www.argenprop.com/departamento-en-venta-en-mendoza-6-ambientes--19595730</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 110,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 84,500) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1762,11 +1758,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>31.6</v>
+        <v>55.7</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1775,22 +1771,22 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>58000</v>
+        <v>148000</v>
       </c>
       <c r="E19" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F19" t="n">
-        <v>580</v>
+        <v>740</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1810,37 +1806,37 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Duplex En Godoy Cruz</t>
+          <t>Departamento en venta c/ cochera en centro</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
+          <t>https://www.argenprop.com/departamento-en-venta-en-mendoza-7-ambientes--19590181</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 58,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>Publicado en USD 148,000 (Requiere contraoferta del 5.7%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>30</v>
+        <v>54.1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1849,22 +1845,22 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>85000</v>
+        <v>99000</v>
       </c>
       <c r="E20" t="n">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="F20" t="n">
-        <v>1133.3</v>
+        <v>1020.6</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1889,32 +1885,32 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>🏡 ¡Viví en una de las zonas más buscadas de Ciudad! 📍 Paso de los Andes N° 570, a 100 metros de Arístides de Villanueva, Ciudad</t>
+          <t>Depto venta duplex 2 dorm cochera</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/133635-di-luca-propiedades/inmuebles/98/ficha/departamento-en-venta-en-paso-de-los-andes-n0-570-ciudad</t>
+          <t>https://www.argenprop.com/departamento-en-venta-en-s1-parque-central-3-ambientes--19531214</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 85,000) | 💡 Publicación indica apertura a ofertas o permutas</t>
+          <t>Dentro del presupuesto (USD 99,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera | 💡 Publicación indica apertura a ofertas o permutas</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>30</v>
+        <v>54.1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1923,13 +1919,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>150000</v>
+        <v>72000</v>
       </c>
       <c r="E21" t="n">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="F21" t="n">
-        <v>1898.7</v>
+        <v>774.2</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1958,52 +1954,52 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Moderada</t>
+          <t>Estándar</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
+          <t>Venta departamento 3 dormitorios – ciudad de mendoza</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
+          <t>https://www.argenprop.com/departamento-en-venta-en-primera-seccion-5-ambientes--19707482</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 72,000) | 🛗 Edificio con ascensor</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>28.5</v>
+        <v>53.5</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Guaymallen</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>90000</v>
+        <v>50000</v>
       </c>
       <c r="E22" t="n">
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="F22" t="n">
-        <v>1000</v>
+        <v>322.6</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2012,7 +2008,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2037,28 +2033,28 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>#Oportunidad de Inversión – Zona Poder Judicial#</t>
+          <t>Vendo casa en dorrego</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/308921-femmestate/inmuebles/133/ficha/departamento-en-venta-en-p-molina-y-mitre</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-coronel-dorrego-3-ambientes--20431316</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000) | 🛗 Edificio con ascensor</t>
+          <t>Dentro del presupuesto (USD 50,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>24.8</v>
+        <v>52.8</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2071,17 +2067,17 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>140000</v>
+        <v>75000</v>
       </c>
       <c r="E23" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F23" t="n">
-        <v>1866.7</v>
+        <v>961.5</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>No/Duda</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2106,52 +2102,52 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Departamento en Venta – Mendoza Capital</t>
+          <t>Departamento tipo dúplex en barrio bancario godoy cruz mendoza</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/276253-sere-inmobiliaria/inmuebles/136/ficha/departamento-en-venta-en-peatonal-y-9-de-julio</t>
+          <t>https://www.argenprop.com/departamento-en-venta-en-godoy-cruz-5-ambientes--20617012</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 75,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>20.9</v>
+        <v>51.5</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>80000</v>
+        <v>150000</v>
       </c>
       <c r="E24" t="n">
-        <v>90</v>
+        <v>220</v>
       </c>
       <c r="F24" t="n">
-        <v>888.9</v>
+        <v>681.8</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2160,7 +2156,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2180,52 +2176,52 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Estándar</t>
+          <t>Moderada</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
+          <t>Casa en b° bombal - apta estudio y oficinas - apta credito</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-mendoza-9-ambientes--19928430</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 80,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>20</v>
+        <v>48.9</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Mendoza</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>90000</v>
+        <v>140000</v>
       </c>
       <c r="E25" t="n">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="F25" t="n">
-        <v>1343.3</v>
+        <v>1538.5</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2234,7 +2230,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2259,28 +2255,28 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>¡Departamento remodelado frente a Plaza España! – 9 de Julio, Planta Baja</t>
+          <t>Duplex frente al dalvian</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://www.inmoclick.com.ar/8993-lombardo-propiedades/inmuebles/136/ficha/departamento-en-venta-en-espana-esq-san-lorenzo</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-mendoza--18669561</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 90,000)</t>
+          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20</v>
+        <v>48.5</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2289,17 +2285,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Departamento</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>75000</v>
+        <v>79000</v>
       </c>
       <c r="E26" t="n">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="F26" t="n">
-        <v>1119.4</v>
+        <v>658.3</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2308,7 +2304,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2333,17 +2329,17 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Departamento En Las Tortugas</t>
+          <t>Casa 500m2 parque hiper libertad</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://departamento.mercadolibre.com.ar/MLA-2133562131-departamento-en-las-tortugas-_JM</t>
+          <t>https://www.argenprop.com/casa-en-venta-en-godoy-cruz-4-ambientes--19742664</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Dentro del presupuesto (USD 75,000)</t>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 79,000) | 🚗 Cuenta con cochera</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2354,73 +2350,2445 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>76000</v>
+      </c>
+      <c r="E27" t="n">
+        <v>117</v>
+      </c>
+      <c r="F27" t="n">
+        <v>649.6</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Vendo casa en barrio san ignacio, godoy cruz</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/casa-en-venta-en-villa-hipodromo-4-ambientes--19442483</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 76,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>85000</v>
+      </c>
+      <c r="E28" t="n">
+        <v>164</v>
+      </c>
+      <c r="F28" t="n">
+        <v>518.3</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Casa en venta - 3 dormitorios, 2 baños, amplio jardín y terraza</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/casa-en-venta-en-villa-hipodromo-6-ambientes--19928448</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 85,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E29" t="n">
+        <v>200</v>
+      </c>
+      <c r="F29" t="n">
+        <v>350</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Casa esquina en 2 planta con salón comercial – godoy cruz</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/casa-en-venta-en-villa-hipodromo-6-ambientes--17029440</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 70,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>48</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>94900</v>
+      </c>
+      <c r="E30" t="n">
+        <v>170</v>
+      </c>
+      <c r="F30" t="n">
+        <v>558.2</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Venta casa en el barrio trapiche de godoy cruz</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/casa-en-venta-en-gobernador-benegas-5-ambientes--19957421</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 94,900) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>78000</v>
+      </c>
+      <c r="E31" t="n">
+        <v>130</v>
+      </c>
+      <c r="F31" t="n">
+        <v>600</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Departamento en venta en centro</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/departamento-en-venta-en-mendoza-6-ambientes--19590129</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 78,000)</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E32" t="n">
+        <v>137</v>
+      </c>
+      <c r="F32" t="n">
+        <v>656.9</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Venta Excelente Departamento Tipo Casa En Mendoza</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1808643353-venta-excelente-departamento-tipo-casa-en-mendoza-_JM</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000)</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>92000</v>
+      </c>
+      <c r="E33" t="n">
+        <v>105</v>
+      </c>
+      <c r="F33" t="n">
+        <v>876.2</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>RE/MAX Follow presenta departamento en venta en Ciudad de Mendoza</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/274909-remax-follow/inmuebles/2549/ficha/departamento-en-venta-en-avenida-san-martin-1000</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 92,000)</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>120000</v>
+      </c>
+      <c r="E34" t="n">
+        <v>150</v>
+      </c>
+      <c r="F34" t="n">
+        <v>800</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>🏢 DEPARTAMENTO EN VENTA – CAPITAL, MENDOZA</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/312047-alvarez-asociados/inmuebles/12/ficha/departamento-en-venta-en-olascoaga-n-o-1566-entre-agustin-alvarez-y-avellaneda</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 120,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>124000</v>
+      </c>
+      <c r="E35" t="n">
+        <v>166</v>
+      </c>
+      <c r="F35" t="n">
+        <v>747</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Casa en venta en san martín sur, godoy cruz</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/casa-en-venta-en-godoy-cruz-5-ambientes--20223446</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 124,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Guaymallen</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>55000</v>
+      </c>
+      <c r="E36" t="n">
+        <v>88</v>
+      </c>
+      <c r="F36" t="n">
+        <v>625</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Venta De Departamento Planta Alta Coronel Dorrego</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2130172827-venta-de-departamento-planta-alta-coronel-dorrego-_JM</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 55,000)</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>53000</v>
+      </c>
+      <c r="E37" t="n">
+        <v>70</v>
+      </c>
+      <c r="F37" t="n">
+        <v>757.1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Planta baja confortable y funcional en excelente zona de Dorrego, entre las calles Laprida y Cobos, adyacencias calle Lamadrid, ideal para quienes buscan comodidad, privacidad y ubicación estratégica. Un hogar pensado para el día a día: living comedor para recibir visitas, cocina comedor práctica para las comidas diarias y una lavandería independiente que facilita las tareas del hogar. Tres dormitorios bien distribuidos: dos con placares y un tercero en suite con su propio placard, que ofrece mayor privacidad y confort.</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/308706-cm/inmuebles/6/ficha/departamento-en-venta-en-laprida-y-cobos</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 53,000)</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>116000</v>
+      </c>
+      <c r="E38" t="n">
+        <v>120</v>
+      </c>
+      <c r="F38" t="n">
+        <v>966.7</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>DEPARTAMENTO EN VENTA</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/29719-martin-helder/inmuebles/34/ficha/departamento-en-venta-en-sarmiento-290</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 116,000) | 🔥 Red de gas natural confirmada</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>44</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>78000</v>
+      </c>
+      <c r="E39" t="n">
+        <v>78</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Vendo departamento en ciudad</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/departamento-en-venta-en-mendoza-4-ambientes--20024054</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 78,000)</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>43</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>89000</v>
+      </c>
+      <c r="E40" t="n">
+        <v>118</v>
+      </c>
+      <c r="F40" t="n">
+        <v>754.2</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>SIGILO DESARROLLOS INMOBILIARIOS VENDE</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/29891-sigilo-desarrollos-inmobiliarios/inmuebles/109/ficha/departamento-en-venta-en-paraguay-y-castelar</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 89,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>139000</v>
+      </c>
+      <c r="E41" t="n">
+        <v>86</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1616.3</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Vendo departamento en barrio bombal. apto credito hipotecario.</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/departamento-en-venta-en-godoy-cruz-4-ambientes--18838233</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>📍 Excelente ubicación: Barrio Bombal / Bombal Sur (Godoy Cruz) | ✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 139,000)</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>42</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>77000</v>
+      </c>
+      <c r="E42" t="n">
+        <v>97</v>
+      </c>
+      <c r="F42" t="n">
+        <v>793.8</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>VENTA DE DEPARTAMENTO DE 3 HABITACIONES CON TERRAZA PROPIA A RECICLAR A METROS DE LA PLAZA ITALIA, MENDOZA.</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/310522-ana-lucia-raina-propiedades/inmuebles/9/ficha/departamento-en-venta-en-peru-y-montevideo</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 77,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>115000</v>
+      </c>
+      <c r="E43" t="n">
+        <v>110</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1045.5</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>FEMMESTATE VENDE Departamento  en plena Ciudad de Mendoza</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/308921-femmestate/inmuebles/178/ficha/departamento-en-venta-en-necochea</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 115,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>N/D</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Casa en venta – barrio fuchs – godoy cruz – apta crédito hipotecario</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/casa-en-venta-en-godoy-cruz-5-ambientes--20067816</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>110000</v>
+      </c>
+      <c r="E45" t="n">
+        <v>117</v>
+      </c>
+      <c r="F45" t="n">
+        <v>940.2</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>ZELTA Inmobiliaria Vendo Departamento en Ciudad de Mendoza.</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/302127-zelta-inmobiliaria/inmuebles/170/ficha/departamento-en-venta-en-general-paz-135</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 110,000) | 🛗 Edificio con ascensor</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E46" t="n">
+        <v>120</v>
+      </c>
+      <c r="F46" t="n">
+        <v>666.7</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Se ofrece a la venta amplio departamento en planta baja, ubicado en una excelente zona del centro de Mendoza, sobre calle España, entre Godoy Cruz y Barcala.</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/287601-garach-gestiones-inmobiliarias/inmuebles/55/ficha/departamento-en-venta-en-espana-1751</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 80,000)</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>74000</v>
+      </c>
+      <c r="E47" t="n">
+        <v>211</v>
+      </c>
+      <c r="F47" t="n">
+        <v>350.7</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Venta de casa con local comercial</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/casa-en-venta-en-godoy-cruz-7-ambientes--18020627</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 74,000)</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>68000</v>
+      </c>
+      <c r="E48" t="n">
+        <v>75</v>
+      </c>
+      <c r="F48" t="n">
+        <v>906.7</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>DRUMMOND NEGOCIOS INMOBILIARIOS VENDE</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/124071-drummond-negocios-inmobiliarios/inmuebles/43/ficha/departamento-en-venta-en-espana-y-gutierrez</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 68,000) | 🔥 Red de gas natural confirmada | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Guaymallen</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>110000</v>
+      </c>
+      <c r="E49" t="n">
+        <v>100</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Departamento En Coronel Dorrego</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3024664484-departamento-en-coronel-dorrego-_JM</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 110,000)</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>58000</v>
+      </c>
+      <c r="E50" t="n">
+        <v>100</v>
+      </c>
+      <c r="F50" t="n">
+        <v>580</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Duplex En Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3846544412-duplex-en-godoy-cruz-_JM</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts) | Dentro del presupuesto (USD 58,000)</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>30</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E51" t="n">
+        <v>79</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1898.7</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Moderada</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Venta - Departamento Apto Airbnb - Green Wave - Financiacion</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-1835271625-venta-departamento-apto-airbnb-green-wave-financiacion-_JM</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>✨ Amplio: cuenta con 3+ dormitorios o 4+ ambientes (+10 pts)</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | Publicado en USD 150,000 (Requiere contraoferta del 7.1%) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E52" t="n">
+        <v>65</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1384.6</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Departamento ubicado en 5° piso de Avenida Pedro Molina, Segunda sección de Capital.</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/105122-helga-kruls-propiedades/inmuebles/121/ficha/departamento-en-venta-en-pedro-molina-461</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 90,000) | 🚗 Cuenta con cochera | 🛗 Edificio con ascensor</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E53" t="n">
+        <v>90</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>#Oportunidad de Inversión – Zona Poder Judicial#</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/308921-femmestate/inmuebles/133/ficha/departamento-en-venta-en-p-molina-y-mitre</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 90,000) | 🛗 Edificio con ascensor</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>83000</v>
+      </c>
+      <c r="E54" t="n">
+        <v>66</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1257.6</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Vendo departamentos y dúplex en lote iv complejo cervantes, godoy cruz</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>https://www.argenprop.com/departamento-en-venta-en-godoy-cruz-3-ambientes--20157226</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 83,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>140000</v>
+      </c>
+      <c r="E55" t="n">
+        <v>75</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1866.7</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Departamento en Venta – Mendoza Capital</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/276253-sere-inmobiliaria/inmuebles/136/ficha/departamento-en-venta-en-peatonal-y-9-de-julio</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 140,000) | 🚗 Cuenta con cochera</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E56" t="n">
+        <v>90</v>
+      </c>
+      <c r="F56" t="n">
+        <v>888.9</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Departamento En Venta - Benegas - Godoy Cruz - Mendoza</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-3756706742-departamento-en-venta-benegas-godoy-cruz-mendoza-_JM</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 80,000)</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
         <v>20</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Godoy Cruz</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Departamento</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D57" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E57" t="n">
+        <v>67</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1343.3</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>¡Departamento remodelado frente a Plaza España! – 9 de Julio, Planta Baja</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>https://www.inmoclick.com.ar/8993-lombardo-propiedades/inmuebles/136/ficha/departamento-en-venta-en-espana-esq-san-lorenzo</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 90,000)</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>20</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E58" t="n">
+        <v>67</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1119.4</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Departamento En Las Tortugas</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>https://departamento.mercadolibre.com.ar/MLA-2133562131-departamento-en-las-tortugas-_JM</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Dentro del presupuesto (USD 75,000)</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>20</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Departamento</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
         <v>63300</v>
       </c>
-      <c r="E27" t="n">
+      <c r="E59" t="n">
         <v>73</v>
       </c>
-      <c r="F27" t="n">
+      <c r="F59" t="n">
         <v>867.1</v>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>No/Duda</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Estándar</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>No/Duda</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
         <is>
           <t>Departamento En Gobernador Benegas</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N59" t="inlineStr">
         <is>
           <t>https://departamento.mercadolibre.com.ar/MLA-1713408519-departamento-en-gobernador-benegas-_JM</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O59" t="inlineStr">
         <is>
           <t>Dentro del presupuesto (USD 63,300)</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P59" t="inlineStr">
         <is>
           <t>⚠️ Ubicado en Godoy Cruz fuera de Barrio Bombal (-15 pts) | ⚠️ Sin seguridad 24 hs ni barrio privado (penalizado en puntaje) | Consultar conexión a red de gas natural</t>
         </is>

</xml_diff>